<commit_message>
Périodicité de facturation, confirmation de suppression, import plus robuste
- Périodicité mensuelle, trimestrielle, semestrielle ou annuelle : par
  défaut dans Réglages, modifiable par client (fiche, tableau, modèle
  Excel, import/export) ; la lettre indique le montant HT et TTC par période.
- Suppression d'un client ou des exemples : demande de confirmation.
- Import : lecture des .xlsx quel que soit le nom ou l'extension,
  balises XML sans préfixe imposé, recherche de la bonne feuille,
  message clair si le modèle ne contient que la ligne d'exemple ou si le
  format (.xls, .ods, .numbers) n'est pas lisible.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016XDuNfo7Y47EZPw7PCgVRg
</commit_message>
<xml_diff>
--- a/Modele_import_clients.xlsx
+++ b/Modele_import_clients.xlsx
@@ -211,10 +211,15 @@
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
+        <t>Mensuelle, Trimestrielle, Semestrielle ou Annuelle. Vide = périodicité par défaut du cabinet.</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
         <t>Oui / Non. Vide = Oui.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Courrier, Email ou Les deux. Vide = Courrier.</t>
       </text>
@@ -512,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P501"/>
+  <dimension ref="A1:Q501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -529,8 +534,9 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -606,10 +612,15 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>Périodicité</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>À envoyer</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Mode d'envoi</t>
         </is>
@@ -676,10 +687,15 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
+          <t>Mensuelle</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Courrier</t>
         </is>
@@ -702,6 +718,7 @@
       <c r="N3" s="7" t="n"/>
       <c r="O3" s="5" t="n"/>
       <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -720,6 +737,7 @@
       <c r="N4" s="7" t="n"/>
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -738,6 +756,7 @@
       <c r="N5" s="7" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -756,6 +775,7 @@
       <c r="N6" s="7" t="n"/>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -774,6 +794,7 @@
       <c r="N7" s="7" t="n"/>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -792,6 +813,7 @@
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -810,6 +832,7 @@
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -828,6 +851,7 @@
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -846,6 +870,7 @@
       <c r="N11" s="7" t="n"/>
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -864,6 +889,7 @@
       <c r="N12" s="7" t="n"/>
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -882,6 +908,7 @@
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -900,6 +927,7 @@
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -918,6 +946,7 @@
       <c r="N15" s="7" t="n"/>
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -936,6 +965,7 @@
       <c r="N16" s="7" t="n"/>
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -954,6 +984,7 @@
       <c r="N17" s="7" t="n"/>
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="5" t="n"/>
+      <c r="Q17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -972,6 +1003,7 @@
       <c r="N18" s="7" t="n"/>
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="5" t="n"/>
+      <c r="Q18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -990,6 +1022,7 @@
       <c r="N19" s="7" t="n"/>
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="5" t="n"/>
+      <c r="Q19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1008,6 +1041,7 @@
       <c r="N20" s="7" t="n"/>
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1026,6 +1060,7 @@
       <c r="N21" s="7" t="n"/>
       <c r="O21" s="5" t="n"/>
       <c r="P21" s="5" t="n"/>
+      <c r="Q21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1044,6 +1079,7 @@
       <c r="N22" s="7" t="n"/>
       <c r="O22" s="5" t="n"/>
       <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1062,6 +1098,7 @@
       <c r="N23" s="7" t="n"/>
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="5" t="n"/>
+      <c r="Q23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1080,6 +1117,7 @@
       <c r="N24" s="7" t="n"/>
       <c r="O24" s="5" t="n"/>
       <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1098,6 +1136,7 @@
       <c r="N25" s="7" t="n"/>
       <c r="O25" s="5" t="n"/>
       <c r="P25" s="5" t="n"/>
+      <c r="Q25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1116,6 +1155,7 @@
       <c r="N26" s="7" t="n"/>
       <c r="O26" s="5" t="n"/>
       <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1134,6 +1174,7 @@
       <c r="N27" s="7" t="n"/>
       <c r="O27" s="5" t="n"/>
       <c r="P27" s="5" t="n"/>
+      <c r="Q27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1152,6 +1193,7 @@
       <c r="N28" s="7" t="n"/>
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1170,6 +1212,7 @@
       <c r="N29" s="7" t="n"/>
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="5" t="n"/>
+      <c r="Q29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1188,6 +1231,7 @@
       <c r="N30" s="7" t="n"/>
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1206,6 +1250,7 @@
       <c r="N31" s="7" t="n"/>
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="5" t="n"/>
+      <c r="Q31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1224,6 +1269,7 @@
       <c r="N32" s="7" t="n"/>
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="5" t="n"/>
+      <c r="Q32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1242,6 +1288,7 @@
       <c r="N33" s="7" t="n"/>
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="5" t="n"/>
+      <c r="Q33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1260,6 +1307,7 @@
       <c r="N34" s="7" t="n"/>
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="5" t="n"/>
+      <c r="Q34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1278,6 +1326,7 @@
       <c r="N35" s="7" t="n"/>
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="5" t="n"/>
+      <c r="Q35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1296,6 +1345,7 @@
       <c r="N36" s="7" t="n"/>
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1314,6 +1364,7 @@
       <c r="N37" s="7" t="n"/>
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="5" t="n"/>
+      <c r="Q37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1332,6 +1383,7 @@
       <c r="N38" s="7" t="n"/>
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="5" t="n"/>
+      <c r="Q38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1350,6 +1402,7 @@
       <c r="N39" s="7" t="n"/>
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="5" t="n"/>
+      <c r="Q39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1368,6 +1421,7 @@
       <c r="N40" s="7" t="n"/>
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="5" t="n"/>
+      <c r="Q40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1386,6 +1440,7 @@
       <c r="N41" s="7" t="n"/>
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="5" t="n"/>
+      <c r="Q41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1404,6 +1459,7 @@
       <c r="N42" s="7" t="n"/>
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="5" t="n"/>
+      <c r="Q42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1422,6 +1478,7 @@
       <c r="N43" s="7" t="n"/>
       <c r="O43" s="5" t="n"/>
       <c r="P43" s="5" t="n"/>
+      <c r="Q43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1440,6 +1497,7 @@
       <c r="N44" s="7" t="n"/>
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="5" t="n"/>
+      <c r="Q44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1458,6 +1516,7 @@
       <c r="N45" s="7" t="n"/>
       <c r="O45" s="5" t="n"/>
       <c r="P45" s="5" t="n"/>
+      <c r="Q45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1476,6 +1535,7 @@
       <c r="N46" s="7" t="n"/>
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="5" t="n"/>
+      <c r="Q46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1494,6 +1554,7 @@
       <c r="N47" s="7" t="n"/>
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="5" t="n"/>
+      <c r="Q47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1512,6 +1573,7 @@
       <c r="N48" s="7" t="n"/>
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="5" t="n"/>
+      <c r="Q48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1530,6 +1592,7 @@
       <c r="N49" s="7" t="n"/>
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="5" t="n"/>
+      <c r="Q49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1548,6 +1611,7 @@
       <c r="N50" s="7" t="n"/>
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="5" t="n"/>
+      <c r="Q50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1566,6 +1630,7 @@
       <c r="N51" s="7" t="n"/>
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="5" t="n"/>
+      <c r="Q51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1584,6 +1649,7 @@
       <c r="N52" s="7" t="n"/>
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="5" t="n"/>
+      <c r="Q52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1602,6 +1668,7 @@
       <c r="N53" s="7" t="n"/>
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="5" t="n"/>
+      <c r="Q53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1620,6 +1687,7 @@
       <c r="N54" s="7" t="n"/>
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="5" t="n"/>
+      <c r="Q54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -1638,6 +1706,7 @@
       <c r="N55" s="7" t="n"/>
       <c r="O55" s="5" t="n"/>
       <c r="P55" s="5" t="n"/>
+      <c r="Q55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -1656,6 +1725,7 @@
       <c r="N56" s="7" t="n"/>
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="5" t="n"/>
+      <c r="Q56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -1674,6 +1744,7 @@
       <c r="N57" s="7" t="n"/>
       <c r="O57" s="5" t="n"/>
       <c r="P57" s="5" t="n"/>
+      <c r="Q57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -1692,6 +1763,7 @@
       <c r="N58" s="7" t="n"/>
       <c r="O58" s="5" t="n"/>
       <c r="P58" s="5" t="n"/>
+      <c r="Q58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -1710,6 +1782,7 @@
       <c r="N59" s="7" t="n"/>
       <c r="O59" s="5" t="n"/>
       <c r="P59" s="5" t="n"/>
+      <c r="Q59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -1728,6 +1801,7 @@
       <c r="N60" s="7" t="n"/>
       <c r="O60" s="5" t="n"/>
       <c r="P60" s="5" t="n"/>
+      <c r="Q60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -1746,6 +1820,7 @@
       <c r="N61" s="7" t="n"/>
       <c r="O61" s="5" t="n"/>
       <c r="P61" s="5" t="n"/>
+      <c r="Q61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -1764,6 +1839,7 @@
       <c r="N62" s="7" t="n"/>
       <c r="O62" s="5" t="n"/>
       <c r="P62" s="5" t="n"/>
+      <c r="Q62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -1782,6 +1858,7 @@
       <c r="N63" s="7" t="n"/>
       <c r="O63" s="5" t="n"/>
       <c r="P63" s="5" t="n"/>
+      <c r="Q63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -1800,6 +1877,7 @@
       <c r="N64" s="7" t="n"/>
       <c r="O64" s="5" t="n"/>
       <c r="P64" s="5" t="n"/>
+      <c r="Q64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -1818,6 +1896,7 @@
       <c r="N65" s="7" t="n"/>
       <c r="O65" s="5" t="n"/>
       <c r="P65" s="5" t="n"/>
+      <c r="Q65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -1836,6 +1915,7 @@
       <c r="N66" s="7" t="n"/>
       <c r="O66" s="5" t="n"/>
       <c r="P66" s="5" t="n"/>
+      <c r="Q66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -1854,6 +1934,7 @@
       <c r="N67" s="7" t="n"/>
       <c r="O67" s="5" t="n"/>
       <c r="P67" s="5" t="n"/>
+      <c r="Q67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -1872,6 +1953,7 @@
       <c r="N68" s="7" t="n"/>
       <c r="O68" s="5" t="n"/>
       <c r="P68" s="5" t="n"/>
+      <c r="Q68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -1890,6 +1972,7 @@
       <c r="N69" s="7" t="n"/>
       <c r="O69" s="5" t="n"/>
       <c r="P69" s="5" t="n"/>
+      <c r="Q69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -1908,6 +1991,7 @@
       <c r="N70" s="7" t="n"/>
       <c r="O70" s="5" t="n"/>
       <c r="P70" s="5" t="n"/>
+      <c r="Q70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -1926,6 +2010,7 @@
       <c r="N71" s="7" t="n"/>
       <c r="O71" s="5" t="n"/>
       <c r="P71" s="5" t="n"/>
+      <c r="Q71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -1944,6 +2029,7 @@
       <c r="N72" s="7" t="n"/>
       <c r="O72" s="5" t="n"/>
       <c r="P72" s="5" t="n"/>
+      <c r="Q72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -1962,6 +2048,7 @@
       <c r="N73" s="7" t="n"/>
       <c r="O73" s="5" t="n"/>
       <c r="P73" s="5" t="n"/>
+      <c r="Q73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -1980,6 +2067,7 @@
       <c r="N74" s="7" t="n"/>
       <c r="O74" s="5" t="n"/>
       <c r="P74" s="5" t="n"/>
+      <c r="Q74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -1998,6 +2086,7 @@
       <c r="N75" s="7" t="n"/>
       <c r="O75" s="5" t="n"/>
       <c r="P75" s="5" t="n"/>
+      <c r="Q75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -2016,6 +2105,7 @@
       <c r="N76" s="7" t="n"/>
       <c r="O76" s="5" t="n"/>
       <c r="P76" s="5" t="n"/>
+      <c r="Q76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -2034,6 +2124,7 @@
       <c r="N77" s="7" t="n"/>
       <c r="O77" s="5" t="n"/>
       <c r="P77" s="5" t="n"/>
+      <c r="Q77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -2052,6 +2143,7 @@
       <c r="N78" s="7" t="n"/>
       <c r="O78" s="5" t="n"/>
       <c r="P78" s="5" t="n"/>
+      <c r="Q78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -2070,6 +2162,7 @@
       <c r="N79" s="7" t="n"/>
       <c r="O79" s="5" t="n"/>
       <c r="P79" s="5" t="n"/>
+      <c r="Q79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -2088,6 +2181,7 @@
       <c r="N80" s="7" t="n"/>
       <c r="O80" s="5" t="n"/>
       <c r="P80" s="5" t="n"/>
+      <c r="Q80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -2106,6 +2200,7 @@
       <c r="N81" s="7" t="n"/>
       <c r="O81" s="5" t="n"/>
       <c r="P81" s="5" t="n"/>
+      <c r="Q81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -2124,6 +2219,7 @@
       <c r="N82" s="7" t="n"/>
       <c r="O82" s="5" t="n"/>
       <c r="P82" s="5" t="n"/>
+      <c r="Q82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -2142,6 +2238,7 @@
       <c r="N83" s="7" t="n"/>
       <c r="O83" s="5" t="n"/>
       <c r="P83" s="5" t="n"/>
+      <c r="Q83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -2160,6 +2257,7 @@
       <c r="N84" s="7" t="n"/>
       <c r="O84" s="5" t="n"/>
       <c r="P84" s="5" t="n"/>
+      <c r="Q84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -2178,6 +2276,7 @@
       <c r="N85" s="7" t="n"/>
       <c r="O85" s="5" t="n"/>
       <c r="P85" s="5" t="n"/>
+      <c r="Q85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -2196,6 +2295,7 @@
       <c r="N86" s="7" t="n"/>
       <c r="O86" s="5" t="n"/>
       <c r="P86" s="5" t="n"/>
+      <c r="Q86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -2214,6 +2314,7 @@
       <c r="N87" s="7" t="n"/>
       <c r="O87" s="5" t="n"/>
       <c r="P87" s="5" t="n"/>
+      <c r="Q87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -2232,6 +2333,7 @@
       <c r="N88" s="7" t="n"/>
       <c r="O88" s="5" t="n"/>
       <c r="P88" s="5" t="n"/>
+      <c r="Q88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -2250,6 +2352,7 @@
       <c r="N89" s="7" t="n"/>
       <c r="O89" s="5" t="n"/>
       <c r="P89" s="5" t="n"/>
+      <c r="Q89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -2268,6 +2371,7 @@
       <c r="N90" s="7" t="n"/>
       <c r="O90" s="5" t="n"/>
       <c r="P90" s="5" t="n"/>
+      <c r="Q90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -2286,6 +2390,7 @@
       <c r="N91" s="7" t="n"/>
       <c r="O91" s="5" t="n"/>
       <c r="P91" s="5" t="n"/>
+      <c r="Q91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -2304,6 +2409,7 @@
       <c r="N92" s="7" t="n"/>
       <c r="O92" s="5" t="n"/>
       <c r="P92" s="5" t="n"/>
+      <c r="Q92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -2322,6 +2428,7 @@
       <c r="N93" s="7" t="n"/>
       <c r="O93" s="5" t="n"/>
       <c r="P93" s="5" t="n"/>
+      <c r="Q93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -2340,6 +2447,7 @@
       <c r="N94" s="7" t="n"/>
       <c r="O94" s="5" t="n"/>
       <c r="P94" s="5" t="n"/>
+      <c r="Q94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -2358,6 +2466,7 @@
       <c r="N95" s="7" t="n"/>
       <c r="O95" s="5" t="n"/>
       <c r="P95" s="5" t="n"/>
+      <c r="Q95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -2376,6 +2485,7 @@
       <c r="N96" s="7" t="n"/>
       <c r="O96" s="5" t="n"/>
       <c r="P96" s="5" t="n"/>
+      <c r="Q96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -2394,6 +2504,7 @@
       <c r="N97" s="7" t="n"/>
       <c r="O97" s="5" t="n"/>
       <c r="P97" s="5" t="n"/>
+      <c r="Q97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -2412,6 +2523,7 @@
       <c r="N98" s="7" t="n"/>
       <c r="O98" s="5" t="n"/>
       <c r="P98" s="5" t="n"/>
+      <c r="Q98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -2430,6 +2542,7 @@
       <c r="N99" s="7" t="n"/>
       <c r="O99" s="5" t="n"/>
       <c r="P99" s="5" t="n"/>
+      <c r="Q99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -2448,6 +2561,7 @@
       <c r="N100" s="7" t="n"/>
       <c r="O100" s="5" t="n"/>
       <c r="P100" s="5" t="n"/>
+      <c r="Q100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -2466,6 +2580,7 @@
       <c r="N101" s="7" t="n"/>
       <c r="O101" s="5" t="n"/>
       <c r="P101" s="5" t="n"/>
+      <c r="Q101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -2484,6 +2599,7 @@
       <c r="N102" s="7" t="n"/>
       <c r="O102" s="5" t="n"/>
       <c r="P102" s="5" t="n"/>
+      <c r="Q102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -2502,6 +2618,7 @@
       <c r="N103" s="7" t="n"/>
       <c r="O103" s="5" t="n"/>
       <c r="P103" s="5" t="n"/>
+      <c r="Q103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -2520,6 +2637,7 @@
       <c r="N104" s="7" t="n"/>
       <c r="O104" s="5" t="n"/>
       <c r="P104" s="5" t="n"/>
+      <c r="Q104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -2538,6 +2656,7 @@
       <c r="N105" s="7" t="n"/>
       <c r="O105" s="5" t="n"/>
       <c r="P105" s="5" t="n"/>
+      <c r="Q105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -2556,6 +2675,7 @@
       <c r="N106" s="7" t="n"/>
       <c r="O106" s="5" t="n"/>
       <c r="P106" s="5" t="n"/>
+      <c r="Q106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -2574,6 +2694,7 @@
       <c r="N107" s="7" t="n"/>
       <c r="O107" s="5" t="n"/>
       <c r="P107" s="5" t="n"/>
+      <c r="Q107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -2592,6 +2713,7 @@
       <c r="N108" s="7" t="n"/>
       <c r="O108" s="5" t="n"/>
       <c r="P108" s="5" t="n"/>
+      <c r="Q108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -2610,6 +2732,7 @@
       <c r="N109" s="7" t="n"/>
       <c r="O109" s="5" t="n"/>
       <c r="P109" s="5" t="n"/>
+      <c r="Q109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -2628,6 +2751,7 @@
       <c r="N110" s="7" t="n"/>
       <c r="O110" s="5" t="n"/>
       <c r="P110" s="5" t="n"/>
+      <c r="Q110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -2646,6 +2770,7 @@
       <c r="N111" s="7" t="n"/>
       <c r="O111" s="5" t="n"/>
       <c r="P111" s="5" t="n"/>
+      <c r="Q111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -2664,6 +2789,7 @@
       <c r="N112" s="7" t="n"/>
       <c r="O112" s="5" t="n"/>
       <c r="P112" s="5" t="n"/>
+      <c r="Q112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -2682,6 +2808,7 @@
       <c r="N113" s="7" t="n"/>
       <c r="O113" s="5" t="n"/>
       <c r="P113" s="5" t="n"/>
+      <c r="Q113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -2700,6 +2827,7 @@
       <c r="N114" s="7" t="n"/>
       <c r="O114" s="5" t="n"/>
       <c r="P114" s="5" t="n"/>
+      <c r="Q114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -2718,6 +2846,7 @@
       <c r="N115" s="7" t="n"/>
       <c r="O115" s="5" t="n"/>
       <c r="P115" s="5" t="n"/>
+      <c r="Q115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -2736,6 +2865,7 @@
       <c r="N116" s="7" t="n"/>
       <c r="O116" s="5" t="n"/>
       <c r="P116" s="5" t="n"/>
+      <c r="Q116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -2754,6 +2884,7 @@
       <c r="N117" s="7" t="n"/>
       <c r="O117" s="5" t="n"/>
       <c r="P117" s="5" t="n"/>
+      <c r="Q117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -2772,6 +2903,7 @@
       <c r="N118" s="7" t="n"/>
       <c r="O118" s="5" t="n"/>
       <c r="P118" s="5" t="n"/>
+      <c r="Q118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -2790,6 +2922,7 @@
       <c r="N119" s="7" t="n"/>
       <c r="O119" s="5" t="n"/>
       <c r="P119" s="5" t="n"/>
+      <c r="Q119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -2808,6 +2941,7 @@
       <c r="N120" s="7" t="n"/>
       <c r="O120" s="5" t="n"/>
       <c r="P120" s="5" t="n"/>
+      <c r="Q120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -2826,6 +2960,7 @@
       <c r="N121" s="7" t="n"/>
       <c r="O121" s="5" t="n"/>
       <c r="P121" s="5" t="n"/>
+      <c r="Q121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -2844,6 +2979,7 @@
       <c r="N122" s="7" t="n"/>
       <c r="O122" s="5" t="n"/>
       <c r="P122" s="5" t="n"/>
+      <c r="Q122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -2862,6 +2998,7 @@
       <c r="N123" s="7" t="n"/>
       <c r="O123" s="5" t="n"/>
       <c r="P123" s="5" t="n"/>
+      <c r="Q123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -2880,6 +3017,7 @@
       <c r="N124" s="7" t="n"/>
       <c r="O124" s="5" t="n"/>
       <c r="P124" s="5" t="n"/>
+      <c r="Q124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -2898,6 +3036,7 @@
       <c r="N125" s="7" t="n"/>
       <c r="O125" s="5" t="n"/>
       <c r="P125" s="5" t="n"/>
+      <c r="Q125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -2916,6 +3055,7 @@
       <c r="N126" s="7" t="n"/>
       <c r="O126" s="5" t="n"/>
       <c r="P126" s="5" t="n"/>
+      <c r="Q126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -2934,6 +3074,7 @@
       <c r="N127" s="7" t="n"/>
       <c r="O127" s="5" t="n"/>
       <c r="P127" s="5" t="n"/>
+      <c r="Q127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -2952,6 +3093,7 @@
       <c r="N128" s="7" t="n"/>
       <c r="O128" s="5" t="n"/>
       <c r="P128" s="5" t="n"/>
+      <c r="Q128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -2970,6 +3112,7 @@
       <c r="N129" s="7" t="n"/>
       <c r="O129" s="5" t="n"/>
       <c r="P129" s="5" t="n"/>
+      <c r="Q129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -2988,6 +3131,7 @@
       <c r="N130" s="7" t="n"/>
       <c r="O130" s="5" t="n"/>
       <c r="P130" s="5" t="n"/>
+      <c r="Q130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -3006,6 +3150,7 @@
       <c r="N131" s="7" t="n"/>
       <c r="O131" s="5" t="n"/>
       <c r="P131" s="5" t="n"/>
+      <c r="Q131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -3024,6 +3169,7 @@
       <c r="N132" s="7" t="n"/>
       <c r="O132" s="5" t="n"/>
       <c r="P132" s="5" t="n"/>
+      <c r="Q132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -3042,6 +3188,7 @@
       <c r="N133" s="7" t="n"/>
       <c r="O133" s="5" t="n"/>
       <c r="P133" s="5" t="n"/>
+      <c r="Q133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -3060,6 +3207,7 @@
       <c r="N134" s="7" t="n"/>
       <c r="O134" s="5" t="n"/>
       <c r="P134" s="5" t="n"/>
+      <c r="Q134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -3078,6 +3226,7 @@
       <c r="N135" s="7" t="n"/>
       <c r="O135" s="5" t="n"/>
       <c r="P135" s="5" t="n"/>
+      <c r="Q135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -3096,6 +3245,7 @@
       <c r="N136" s="7" t="n"/>
       <c r="O136" s="5" t="n"/>
       <c r="P136" s="5" t="n"/>
+      <c r="Q136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -3114,6 +3264,7 @@
       <c r="N137" s="7" t="n"/>
       <c r="O137" s="5" t="n"/>
       <c r="P137" s="5" t="n"/>
+      <c r="Q137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -3132,6 +3283,7 @@
       <c r="N138" s="7" t="n"/>
       <c r="O138" s="5" t="n"/>
       <c r="P138" s="5" t="n"/>
+      <c r="Q138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -3150,6 +3302,7 @@
       <c r="N139" s="7" t="n"/>
       <c r="O139" s="5" t="n"/>
       <c r="P139" s="5" t="n"/>
+      <c r="Q139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -3168,6 +3321,7 @@
       <c r="N140" s="7" t="n"/>
       <c r="O140" s="5" t="n"/>
       <c r="P140" s="5" t="n"/>
+      <c r="Q140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -3186,6 +3340,7 @@
       <c r="N141" s="7" t="n"/>
       <c r="O141" s="5" t="n"/>
       <c r="P141" s="5" t="n"/>
+      <c r="Q141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -3204,6 +3359,7 @@
       <c r="N142" s="7" t="n"/>
       <c r="O142" s="5" t="n"/>
       <c r="P142" s="5" t="n"/>
+      <c r="Q142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -3222,6 +3378,7 @@
       <c r="N143" s="7" t="n"/>
       <c r="O143" s="5" t="n"/>
       <c r="P143" s="5" t="n"/>
+      <c r="Q143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -3240,6 +3397,7 @@
       <c r="N144" s="7" t="n"/>
       <c r="O144" s="5" t="n"/>
       <c r="P144" s="5" t="n"/>
+      <c r="Q144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -3258,6 +3416,7 @@
       <c r="N145" s="7" t="n"/>
       <c r="O145" s="5" t="n"/>
       <c r="P145" s="5" t="n"/>
+      <c r="Q145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -3276,6 +3435,7 @@
       <c r="N146" s="7" t="n"/>
       <c r="O146" s="5" t="n"/>
       <c r="P146" s="5" t="n"/>
+      <c r="Q146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -3294,6 +3454,7 @@
       <c r="N147" s="7" t="n"/>
       <c r="O147" s="5" t="n"/>
       <c r="P147" s="5" t="n"/>
+      <c r="Q147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -3312,6 +3473,7 @@
       <c r="N148" s="7" t="n"/>
       <c r="O148" s="5" t="n"/>
       <c r="P148" s="5" t="n"/>
+      <c r="Q148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -3330,6 +3492,7 @@
       <c r="N149" s="7" t="n"/>
       <c r="O149" s="5" t="n"/>
       <c r="P149" s="5" t="n"/>
+      <c r="Q149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -3348,6 +3511,7 @@
       <c r="N150" s="7" t="n"/>
       <c r="O150" s="5" t="n"/>
       <c r="P150" s="5" t="n"/>
+      <c r="Q150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -3366,6 +3530,7 @@
       <c r="N151" s="7" t="n"/>
       <c r="O151" s="5" t="n"/>
       <c r="P151" s="5" t="n"/>
+      <c r="Q151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -3384,6 +3549,7 @@
       <c r="N152" s="7" t="n"/>
       <c r="O152" s="5" t="n"/>
       <c r="P152" s="5" t="n"/>
+      <c r="Q152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -3402,6 +3568,7 @@
       <c r="N153" s="7" t="n"/>
       <c r="O153" s="5" t="n"/>
       <c r="P153" s="5" t="n"/>
+      <c r="Q153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -3420,6 +3587,7 @@
       <c r="N154" s="7" t="n"/>
       <c r="O154" s="5" t="n"/>
       <c r="P154" s="5" t="n"/>
+      <c r="Q154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -3438,6 +3606,7 @@
       <c r="N155" s="7" t="n"/>
       <c r="O155" s="5" t="n"/>
       <c r="P155" s="5" t="n"/>
+      <c r="Q155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -3456,6 +3625,7 @@
       <c r="N156" s="7" t="n"/>
       <c r="O156" s="5" t="n"/>
       <c r="P156" s="5" t="n"/>
+      <c r="Q156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -3474,6 +3644,7 @@
       <c r="N157" s="7" t="n"/>
       <c r="O157" s="5" t="n"/>
       <c r="P157" s="5" t="n"/>
+      <c r="Q157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -3492,6 +3663,7 @@
       <c r="N158" s="7" t="n"/>
       <c r="O158" s="5" t="n"/>
       <c r="P158" s="5" t="n"/>
+      <c r="Q158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -3510,6 +3682,7 @@
       <c r="N159" s="7" t="n"/>
       <c r="O159" s="5" t="n"/>
       <c r="P159" s="5" t="n"/>
+      <c r="Q159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -3528,6 +3701,7 @@
       <c r="N160" s="7" t="n"/>
       <c r="O160" s="5" t="n"/>
       <c r="P160" s="5" t="n"/>
+      <c r="Q160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -3546,6 +3720,7 @@
       <c r="N161" s="7" t="n"/>
       <c r="O161" s="5" t="n"/>
       <c r="P161" s="5" t="n"/>
+      <c r="Q161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -3564,6 +3739,7 @@
       <c r="N162" s="7" t="n"/>
       <c r="O162" s="5" t="n"/>
       <c r="P162" s="5" t="n"/>
+      <c r="Q162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -3582,6 +3758,7 @@
       <c r="N163" s="7" t="n"/>
       <c r="O163" s="5" t="n"/>
       <c r="P163" s="5" t="n"/>
+      <c r="Q163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -3600,6 +3777,7 @@
       <c r="N164" s="7" t="n"/>
       <c r="O164" s="5" t="n"/>
       <c r="P164" s="5" t="n"/>
+      <c r="Q164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -3618,6 +3796,7 @@
       <c r="N165" s="7" t="n"/>
       <c r="O165" s="5" t="n"/>
       <c r="P165" s="5" t="n"/>
+      <c r="Q165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -3636,6 +3815,7 @@
       <c r="N166" s="7" t="n"/>
       <c r="O166" s="5" t="n"/>
       <c r="P166" s="5" t="n"/>
+      <c r="Q166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -3654,6 +3834,7 @@
       <c r="N167" s="7" t="n"/>
       <c r="O167" s="5" t="n"/>
       <c r="P167" s="5" t="n"/>
+      <c r="Q167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -3672,6 +3853,7 @@
       <c r="N168" s="7" t="n"/>
       <c r="O168" s="5" t="n"/>
       <c r="P168" s="5" t="n"/>
+      <c r="Q168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -3690,6 +3872,7 @@
       <c r="N169" s="7" t="n"/>
       <c r="O169" s="5" t="n"/>
       <c r="P169" s="5" t="n"/>
+      <c r="Q169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -3708,6 +3891,7 @@
       <c r="N170" s="7" t="n"/>
       <c r="O170" s="5" t="n"/>
       <c r="P170" s="5" t="n"/>
+      <c r="Q170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -3726,6 +3910,7 @@
       <c r="N171" s="7" t="n"/>
       <c r="O171" s="5" t="n"/>
       <c r="P171" s="5" t="n"/>
+      <c r="Q171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -3744,6 +3929,7 @@
       <c r="N172" s="7" t="n"/>
       <c r="O172" s="5" t="n"/>
       <c r="P172" s="5" t="n"/>
+      <c r="Q172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -3762,6 +3948,7 @@
       <c r="N173" s="7" t="n"/>
       <c r="O173" s="5" t="n"/>
       <c r="P173" s="5" t="n"/>
+      <c r="Q173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -3780,6 +3967,7 @@
       <c r="N174" s="7" t="n"/>
       <c r="O174" s="5" t="n"/>
       <c r="P174" s="5" t="n"/>
+      <c r="Q174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -3798,6 +3986,7 @@
       <c r="N175" s="7" t="n"/>
       <c r="O175" s="5" t="n"/>
       <c r="P175" s="5" t="n"/>
+      <c r="Q175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -3816,6 +4005,7 @@
       <c r="N176" s="7" t="n"/>
       <c r="O176" s="5" t="n"/>
       <c r="P176" s="5" t="n"/>
+      <c r="Q176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -3834,6 +4024,7 @@
       <c r="N177" s="7" t="n"/>
       <c r="O177" s="5" t="n"/>
       <c r="P177" s="5" t="n"/>
+      <c r="Q177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -3852,6 +4043,7 @@
       <c r="N178" s="7" t="n"/>
       <c r="O178" s="5" t="n"/>
       <c r="P178" s="5" t="n"/>
+      <c r="Q178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -3870,6 +4062,7 @@
       <c r="N179" s="7" t="n"/>
       <c r="O179" s="5" t="n"/>
       <c r="P179" s="5" t="n"/>
+      <c r="Q179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -3888,6 +4081,7 @@
       <c r="N180" s="7" t="n"/>
       <c r="O180" s="5" t="n"/>
       <c r="P180" s="5" t="n"/>
+      <c r="Q180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -3906,6 +4100,7 @@
       <c r="N181" s="7" t="n"/>
       <c r="O181" s="5" t="n"/>
       <c r="P181" s="5" t="n"/>
+      <c r="Q181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -3924,6 +4119,7 @@
       <c r="N182" s="7" t="n"/>
       <c r="O182" s="5" t="n"/>
       <c r="P182" s="5" t="n"/>
+      <c r="Q182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -3942,6 +4138,7 @@
       <c r="N183" s="7" t="n"/>
       <c r="O183" s="5" t="n"/>
       <c r="P183" s="5" t="n"/>
+      <c r="Q183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -3960,6 +4157,7 @@
       <c r="N184" s="7" t="n"/>
       <c r="O184" s="5" t="n"/>
       <c r="P184" s="5" t="n"/>
+      <c r="Q184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -3978,6 +4176,7 @@
       <c r="N185" s="7" t="n"/>
       <c r="O185" s="5" t="n"/>
       <c r="P185" s="5" t="n"/>
+      <c r="Q185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -3996,6 +4195,7 @@
       <c r="N186" s="7" t="n"/>
       <c r="O186" s="5" t="n"/>
       <c r="P186" s="5" t="n"/>
+      <c r="Q186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -4014,6 +4214,7 @@
       <c r="N187" s="7" t="n"/>
       <c r="O187" s="5" t="n"/>
       <c r="P187" s="5" t="n"/>
+      <c r="Q187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -4032,6 +4233,7 @@
       <c r="N188" s="7" t="n"/>
       <c r="O188" s="5" t="n"/>
       <c r="P188" s="5" t="n"/>
+      <c r="Q188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -4050,6 +4252,7 @@
       <c r="N189" s="7" t="n"/>
       <c r="O189" s="5" t="n"/>
       <c r="P189" s="5" t="n"/>
+      <c r="Q189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -4068,6 +4271,7 @@
       <c r="N190" s="7" t="n"/>
       <c r="O190" s="5" t="n"/>
       <c r="P190" s="5" t="n"/>
+      <c r="Q190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -4086,6 +4290,7 @@
       <c r="N191" s="7" t="n"/>
       <c r="O191" s="5" t="n"/>
       <c r="P191" s="5" t="n"/>
+      <c r="Q191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -4104,6 +4309,7 @@
       <c r="N192" s="7" t="n"/>
       <c r="O192" s="5" t="n"/>
       <c r="P192" s="5" t="n"/>
+      <c r="Q192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -4122,6 +4328,7 @@
       <c r="N193" s="7" t="n"/>
       <c r="O193" s="5" t="n"/>
       <c r="P193" s="5" t="n"/>
+      <c r="Q193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -4140,6 +4347,7 @@
       <c r="N194" s="7" t="n"/>
       <c r="O194" s="5" t="n"/>
       <c r="P194" s="5" t="n"/>
+      <c r="Q194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -4158,6 +4366,7 @@
       <c r="N195" s="7" t="n"/>
       <c r="O195" s="5" t="n"/>
       <c r="P195" s="5" t="n"/>
+      <c r="Q195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -4176,6 +4385,7 @@
       <c r="N196" s="7" t="n"/>
       <c r="O196" s="5" t="n"/>
       <c r="P196" s="5" t="n"/>
+      <c r="Q196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -4194,6 +4404,7 @@
       <c r="N197" s="7" t="n"/>
       <c r="O197" s="5" t="n"/>
       <c r="P197" s="5" t="n"/>
+      <c r="Q197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -4212,6 +4423,7 @@
       <c r="N198" s="7" t="n"/>
       <c r="O198" s="5" t="n"/>
       <c r="P198" s="5" t="n"/>
+      <c r="Q198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -4230,6 +4442,7 @@
       <c r="N199" s="7" t="n"/>
       <c r="O199" s="5" t="n"/>
       <c r="P199" s="5" t="n"/>
+      <c r="Q199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -4248,6 +4461,7 @@
       <c r="N200" s="7" t="n"/>
       <c r="O200" s="5" t="n"/>
       <c r="P200" s="5" t="n"/>
+      <c r="Q200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n"/>
@@ -4266,6 +4480,7 @@
       <c r="N201" s="7" t="n"/>
       <c r="O201" s="5" t="n"/>
       <c r="P201" s="5" t="n"/>
+      <c r="Q201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n"/>
@@ -4284,6 +4499,7 @@
       <c r="N202" s="7" t="n"/>
       <c r="O202" s="5" t="n"/>
       <c r="P202" s="5" t="n"/>
+      <c r="Q202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="5" t="n"/>
@@ -4302,6 +4518,7 @@
       <c r="N203" s="7" t="n"/>
       <c r="O203" s="5" t="n"/>
       <c r="P203" s="5" t="n"/>
+      <c r="Q203" s="5" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="5" t="n"/>
@@ -4320,6 +4537,7 @@
       <c r="N204" s="7" t="n"/>
       <c r="O204" s="5" t="n"/>
       <c r="P204" s="5" t="n"/>
+      <c r="Q204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="5" t="n"/>
@@ -4338,6 +4556,7 @@
       <c r="N205" s="7" t="n"/>
       <c r="O205" s="5" t="n"/>
       <c r="P205" s="5" t="n"/>
+      <c r="Q205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="5" t="n"/>
@@ -4356,6 +4575,7 @@
       <c r="N206" s="7" t="n"/>
       <c r="O206" s="5" t="n"/>
       <c r="P206" s="5" t="n"/>
+      <c r="Q206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="5" t="n"/>
@@ -4374,6 +4594,7 @@
       <c r="N207" s="7" t="n"/>
       <c r="O207" s="5" t="n"/>
       <c r="P207" s="5" t="n"/>
+      <c r="Q207" s="5" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="5" t="n"/>
@@ -4392,6 +4613,7 @@
       <c r="N208" s="7" t="n"/>
       <c r="O208" s="5" t="n"/>
       <c r="P208" s="5" t="n"/>
+      <c r="Q208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="5" t="n"/>
@@ -4410,6 +4632,7 @@
       <c r="N209" s="7" t="n"/>
       <c r="O209" s="5" t="n"/>
       <c r="P209" s="5" t="n"/>
+      <c r="Q209" s="5" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="5" t="n"/>
@@ -4428,6 +4651,7 @@
       <c r="N210" s="7" t="n"/>
       <c r="O210" s="5" t="n"/>
       <c r="P210" s="5" t="n"/>
+      <c r="Q210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="5" t="n"/>
@@ -4446,6 +4670,7 @@
       <c r="N211" s="7" t="n"/>
       <c r="O211" s="5" t="n"/>
       <c r="P211" s="5" t="n"/>
+      <c r="Q211" s="5" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="5" t="n"/>
@@ -4464,6 +4689,7 @@
       <c r="N212" s="7" t="n"/>
       <c r="O212" s="5" t="n"/>
       <c r="P212" s="5" t="n"/>
+      <c r="Q212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="5" t="n"/>
@@ -4482,6 +4708,7 @@
       <c r="N213" s="7" t="n"/>
       <c r="O213" s="5" t="n"/>
       <c r="P213" s="5" t="n"/>
+      <c r="Q213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="5" t="n"/>
@@ -4500,6 +4727,7 @@
       <c r="N214" s="7" t="n"/>
       <c r="O214" s="5" t="n"/>
       <c r="P214" s="5" t="n"/>
+      <c r="Q214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="5" t="n"/>
@@ -4518,6 +4746,7 @@
       <c r="N215" s="7" t="n"/>
       <c r="O215" s="5" t="n"/>
       <c r="P215" s="5" t="n"/>
+      <c r="Q215" s="5" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="5" t="n"/>
@@ -4536,6 +4765,7 @@
       <c r="N216" s="7" t="n"/>
       <c r="O216" s="5" t="n"/>
       <c r="P216" s="5" t="n"/>
+      <c r="Q216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="5" t="n"/>
@@ -4554,6 +4784,7 @@
       <c r="N217" s="7" t="n"/>
       <c r="O217" s="5" t="n"/>
       <c r="P217" s="5" t="n"/>
+      <c r="Q217" s="5" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="5" t="n"/>
@@ -4572,6 +4803,7 @@
       <c r="N218" s="7" t="n"/>
       <c r="O218" s="5" t="n"/>
       <c r="P218" s="5" t="n"/>
+      <c r="Q218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="5" t="n"/>
@@ -4590,6 +4822,7 @@
       <c r="N219" s="7" t="n"/>
       <c r="O219" s="5" t="n"/>
       <c r="P219" s="5" t="n"/>
+      <c r="Q219" s="5" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="5" t="n"/>
@@ -4608,6 +4841,7 @@
       <c r="N220" s="7" t="n"/>
       <c r="O220" s="5" t="n"/>
       <c r="P220" s="5" t="n"/>
+      <c r="Q220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="5" t="n"/>
@@ -4626,6 +4860,7 @@
       <c r="N221" s="7" t="n"/>
       <c r="O221" s="5" t="n"/>
       <c r="P221" s="5" t="n"/>
+      <c r="Q221" s="5" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="5" t="n"/>
@@ -4644,6 +4879,7 @@
       <c r="N222" s="7" t="n"/>
       <c r="O222" s="5" t="n"/>
       <c r="P222" s="5" t="n"/>
+      <c r="Q222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="5" t="n"/>
@@ -4662,6 +4898,7 @@
       <c r="N223" s="7" t="n"/>
       <c r="O223" s="5" t="n"/>
       <c r="P223" s="5" t="n"/>
+      <c r="Q223" s="5" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="5" t="n"/>
@@ -4680,6 +4917,7 @@
       <c r="N224" s="7" t="n"/>
       <c r="O224" s="5" t="n"/>
       <c r="P224" s="5" t="n"/>
+      <c r="Q224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="5" t="n"/>
@@ -4698,6 +4936,7 @@
       <c r="N225" s="7" t="n"/>
       <c r="O225" s="5" t="n"/>
       <c r="P225" s="5" t="n"/>
+      <c r="Q225" s="5" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="5" t="n"/>
@@ -4716,6 +4955,7 @@
       <c r="N226" s="7" t="n"/>
       <c r="O226" s="5" t="n"/>
       <c r="P226" s="5" t="n"/>
+      <c r="Q226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="5" t="n"/>
@@ -4734,6 +4974,7 @@
       <c r="N227" s="7" t="n"/>
       <c r="O227" s="5" t="n"/>
       <c r="P227" s="5" t="n"/>
+      <c r="Q227" s="5" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="5" t="n"/>
@@ -4752,6 +4993,7 @@
       <c r="N228" s="7" t="n"/>
       <c r="O228" s="5" t="n"/>
       <c r="P228" s="5" t="n"/>
+      <c r="Q228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n"/>
@@ -4770,6 +5012,7 @@
       <c r="N229" s="7" t="n"/>
       <c r="O229" s="5" t="n"/>
       <c r="P229" s="5" t="n"/>
+      <c r="Q229" s="5" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="5" t="n"/>
@@ -4788,6 +5031,7 @@
       <c r="N230" s="7" t="n"/>
       <c r="O230" s="5" t="n"/>
       <c r="P230" s="5" t="n"/>
+      <c r="Q230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="5" t="n"/>
@@ -4806,6 +5050,7 @@
       <c r="N231" s="7" t="n"/>
       <c r="O231" s="5" t="n"/>
       <c r="P231" s="5" t="n"/>
+      <c r="Q231" s="5" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="5" t="n"/>
@@ -4824,6 +5069,7 @@
       <c r="N232" s="7" t="n"/>
       <c r="O232" s="5" t="n"/>
       <c r="P232" s="5" t="n"/>
+      <c r="Q232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n"/>
@@ -4842,6 +5088,7 @@
       <c r="N233" s="7" t="n"/>
       <c r="O233" s="5" t="n"/>
       <c r="P233" s="5" t="n"/>
+      <c r="Q233" s="5" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n"/>
@@ -4860,6 +5107,7 @@
       <c r="N234" s="7" t="n"/>
       <c r="O234" s="5" t="n"/>
       <c r="P234" s="5" t="n"/>
+      <c r="Q234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="5" t="n"/>
@@ -4878,6 +5126,7 @@
       <c r="N235" s="7" t="n"/>
       <c r="O235" s="5" t="n"/>
       <c r="P235" s="5" t="n"/>
+      <c r="Q235" s="5" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="5" t="n"/>
@@ -4896,6 +5145,7 @@
       <c r="N236" s="7" t="n"/>
       <c r="O236" s="5" t="n"/>
       <c r="P236" s="5" t="n"/>
+      <c r="Q236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="5" t="n"/>
@@ -4914,6 +5164,7 @@
       <c r="N237" s="7" t="n"/>
       <c r="O237" s="5" t="n"/>
       <c r="P237" s="5" t="n"/>
+      <c r="Q237" s="5" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="5" t="n"/>
@@ -4932,6 +5183,7 @@
       <c r="N238" s="7" t="n"/>
       <c r="O238" s="5" t="n"/>
       <c r="P238" s="5" t="n"/>
+      <c r="Q238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n"/>
@@ -4950,6 +5202,7 @@
       <c r="N239" s="7" t="n"/>
       <c r="O239" s="5" t="n"/>
       <c r="P239" s="5" t="n"/>
+      <c r="Q239" s="5" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="5" t="n"/>
@@ -4968,6 +5221,7 @@
       <c r="N240" s="7" t="n"/>
       <c r="O240" s="5" t="n"/>
       <c r="P240" s="5" t="n"/>
+      <c r="Q240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="5" t="n"/>
@@ -4986,6 +5240,7 @@
       <c r="N241" s="7" t="n"/>
       <c r="O241" s="5" t="n"/>
       <c r="P241" s="5" t="n"/>
+      <c r="Q241" s="5" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="n"/>
@@ -5004,6 +5259,7 @@
       <c r="N242" s="7" t="n"/>
       <c r="O242" s="5" t="n"/>
       <c r="P242" s="5" t="n"/>
+      <c r="Q242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="n"/>
@@ -5022,6 +5278,7 @@
       <c r="N243" s="7" t="n"/>
       <c r="O243" s="5" t="n"/>
       <c r="P243" s="5" t="n"/>
+      <c r="Q243" s="5" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="5" t="n"/>
@@ -5040,6 +5297,7 @@
       <c r="N244" s="7" t="n"/>
       <c r="O244" s="5" t="n"/>
       <c r="P244" s="5" t="n"/>
+      <c r="Q244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="5" t="n"/>
@@ -5058,6 +5316,7 @@
       <c r="N245" s="7" t="n"/>
       <c r="O245" s="5" t="n"/>
       <c r="P245" s="5" t="n"/>
+      <c r="Q245" s="5" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="5" t="n"/>
@@ -5076,6 +5335,7 @@
       <c r="N246" s="7" t="n"/>
       <c r="O246" s="5" t="n"/>
       <c r="P246" s="5" t="n"/>
+      <c r="Q246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="5" t="n"/>
@@ -5094,6 +5354,7 @@
       <c r="N247" s="7" t="n"/>
       <c r="O247" s="5" t="n"/>
       <c r="P247" s="5" t="n"/>
+      <c r="Q247" s="5" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n"/>
@@ -5112,6 +5373,7 @@
       <c r="N248" s="7" t="n"/>
       <c r="O248" s="5" t="n"/>
       <c r="P248" s="5" t="n"/>
+      <c r="Q248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="5" t="n"/>
@@ -5130,6 +5392,7 @@
       <c r="N249" s="7" t="n"/>
       <c r="O249" s="5" t="n"/>
       <c r="P249" s="5" t="n"/>
+      <c r="Q249" s="5" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="5" t="n"/>
@@ -5148,6 +5411,7 @@
       <c r="N250" s="7" t="n"/>
       <c r="O250" s="5" t="n"/>
       <c r="P250" s="5" t="n"/>
+      <c r="Q250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="5" t="n"/>
@@ -5166,6 +5430,7 @@
       <c r="N251" s="7" t="n"/>
       <c r="O251" s="5" t="n"/>
       <c r="P251" s="5" t="n"/>
+      <c r="Q251" s="5" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="5" t="n"/>
@@ -5184,6 +5449,7 @@
       <c r="N252" s="7" t="n"/>
       <c r="O252" s="5" t="n"/>
       <c r="P252" s="5" t="n"/>
+      <c r="Q252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="5" t="n"/>
@@ -5202,6 +5468,7 @@
       <c r="N253" s="7" t="n"/>
       <c r="O253" s="5" t="n"/>
       <c r="P253" s="5" t="n"/>
+      <c r="Q253" s="5" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="5" t="n"/>
@@ -5220,6 +5487,7 @@
       <c r="N254" s="7" t="n"/>
       <c r="O254" s="5" t="n"/>
       <c r="P254" s="5" t="n"/>
+      <c r="Q254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="5" t="n"/>
@@ -5238,6 +5506,7 @@
       <c r="N255" s="7" t="n"/>
       <c r="O255" s="5" t="n"/>
       <c r="P255" s="5" t="n"/>
+      <c r="Q255" s="5" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="5" t="n"/>
@@ -5256,6 +5525,7 @@
       <c r="N256" s="7" t="n"/>
       <c r="O256" s="5" t="n"/>
       <c r="P256" s="5" t="n"/>
+      <c r="Q256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n"/>
@@ -5274,6 +5544,7 @@
       <c r="N257" s="7" t="n"/>
       <c r="O257" s="5" t="n"/>
       <c r="P257" s="5" t="n"/>
+      <c r="Q257" s="5" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="5" t="n"/>
@@ -5292,6 +5563,7 @@
       <c r="N258" s="7" t="n"/>
       <c r="O258" s="5" t="n"/>
       <c r="P258" s="5" t="n"/>
+      <c r="Q258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="5" t="n"/>
@@ -5310,6 +5582,7 @@
       <c r="N259" s="7" t="n"/>
       <c r="O259" s="5" t="n"/>
       <c r="P259" s="5" t="n"/>
+      <c r="Q259" s="5" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="5" t="n"/>
@@ -5328,6 +5601,7 @@
       <c r="N260" s="7" t="n"/>
       <c r="O260" s="5" t="n"/>
       <c r="P260" s="5" t="n"/>
+      <c r="Q260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="5" t="n"/>
@@ -5346,6 +5620,7 @@
       <c r="N261" s="7" t="n"/>
       <c r="O261" s="5" t="n"/>
       <c r="P261" s="5" t="n"/>
+      <c r="Q261" s="5" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="5" t="n"/>
@@ -5364,6 +5639,7 @@
       <c r="N262" s="7" t="n"/>
       <c r="O262" s="5" t="n"/>
       <c r="P262" s="5" t="n"/>
+      <c r="Q262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="5" t="n"/>
@@ -5382,6 +5658,7 @@
       <c r="N263" s="7" t="n"/>
       <c r="O263" s="5" t="n"/>
       <c r="P263" s="5" t="n"/>
+      <c r="Q263" s="5" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="5" t="n"/>
@@ -5400,6 +5677,7 @@
       <c r="N264" s="7" t="n"/>
       <c r="O264" s="5" t="n"/>
       <c r="P264" s="5" t="n"/>
+      <c r="Q264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="5" t="n"/>
@@ -5418,6 +5696,7 @@
       <c r="N265" s="7" t="n"/>
       <c r="O265" s="5" t="n"/>
       <c r="P265" s="5" t="n"/>
+      <c r="Q265" s="5" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="5" t="n"/>
@@ -5436,6 +5715,7 @@
       <c r="N266" s="7" t="n"/>
       <c r="O266" s="5" t="n"/>
       <c r="P266" s="5" t="n"/>
+      <c r="Q266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="5" t="n"/>
@@ -5454,6 +5734,7 @@
       <c r="N267" s="7" t="n"/>
       <c r="O267" s="5" t="n"/>
       <c r="P267" s="5" t="n"/>
+      <c r="Q267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="n"/>
@@ -5472,6 +5753,7 @@
       <c r="N268" s="7" t="n"/>
       <c r="O268" s="5" t="n"/>
       <c r="P268" s="5" t="n"/>
+      <c r="Q268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="5" t="n"/>
@@ -5490,6 +5772,7 @@
       <c r="N269" s="7" t="n"/>
       <c r="O269" s="5" t="n"/>
       <c r="P269" s="5" t="n"/>
+      <c r="Q269" s="5" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="5" t="n"/>
@@ -5508,6 +5791,7 @@
       <c r="N270" s="7" t="n"/>
       <c r="O270" s="5" t="n"/>
       <c r="P270" s="5" t="n"/>
+      <c r="Q270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="5" t="n"/>
@@ -5526,6 +5810,7 @@
       <c r="N271" s="7" t="n"/>
       <c r="O271" s="5" t="n"/>
       <c r="P271" s="5" t="n"/>
+      <c r="Q271" s="5" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="5" t="n"/>
@@ -5544,6 +5829,7 @@
       <c r="N272" s="7" t="n"/>
       <c r="O272" s="5" t="n"/>
       <c r="P272" s="5" t="n"/>
+      <c r="Q272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="5" t="n"/>
@@ -5562,6 +5848,7 @@
       <c r="N273" s="7" t="n"/>
       <c r="O273" s="5" t="n"/>
       <c r="P273" s="5" t="n"/>
+      <c r="Q273" s="5" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="5" t="n"/>
@@ -5580,6 +5867,7 @@
       <c r="N274" s="7" t="n"/>
       <c r="O274" s="5" t="n"/>
       <c r="P274" s="5" t="n"/>
+      <c r="Q274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="5" t="n"/>
@@ -5598,6 +5886,7 @@
       <c r="N275" s="7" t="n"/>
       <c r="O275" s="5" t="n"/>
       <c r="P275" s="5" t="n"/>
+      <c r="Q275" s="5" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="5" t="n"/>
@@ -5616,6 +5905,7 @@
       <c r="N276" s="7" t="n"/>
       <c r="O276" s="5" t="n"/>
       <c r="P276" s="5" t="n"/>
+      <c r="Q276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="5" t="n"/>
@@ -5634,6 +5924,7 @@
       <c r="N277" s="7" t="n"/>
       <c r="O277" s="5" t="n"/>
       <c r="P277" s="5" t="n"/>
+      <c r="Q277" s="5" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="5" t="n"/>
@@ -5652,6 +5943,7 @@
       <c r="N278" s="7" t="n"/>
       <c r="O278" s="5" t="n"/>
       <c r="P278" s="5" t="n"/>
+      <c r="Q278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="5" t="n"/>
@@ -5670,6 +5962,7 @@
       <c r="N279" s="7" t="n"/>
       <c r="O279" s="5" t="n"/>
       <c r="P279" s="5" t="n"/>
+      <c r="Q279" s="5" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="5" t="n"/>
@@ -5688,6 +5981,7 @@
       <c r="N280" s="7" t="n"/>
       <c r="O280" s="5" t="n"/>
       <c r="P280" s="5" t="n"/>
+      <c r="Q280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="5" t="n"/>
@@ -5706,6 +6000,7 @@
       <c r="N281" s="7" t="n"/>
       <c r="O281" s="5" t="n"/>
       <c r="P281" s="5" t="n"/>
+      <c r="Q281" s="5" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="5" t="n"/>
@@ -5724,6 +6019,7 @@
       <c r="N282" s="7" t="n"/>
       <c r="O282" s="5" t="n"/>
       <c r="P282" s="5" t="n"/>
+      <c r="Q282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="5" t="n"/>
@@ -5742,6 +6038,7 @@
       <c r="N283" s="7" t="n"/>
       <c r="O283" s="5" t="n"/>
       <c r="P283" s="5" t="n"/>
+      <c r="Q283" s="5" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="5" t="n"/>
@@ -5760,6 +6057,7 @@
       <c r="N284" s="7" t="n"/>
       <c r="O284" s="5" t="n"/>
       <c r="P284" s="5" t="n"/>
+      <c r="Q284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="5" t="n"/>
@@ -5778,6 +6076,7 @@
       <c r="N285" s="7" t="n"/>
       <c r="O285" s="5" t="n"/>
       <c r="P285" s="5" t="n"/>
+      <c r="Q285" s="5" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="5" t="n"/>
@@ -5796,6 +6095,7 @@
       <c r="N286" s="7" t="n"/>
       <c r="O286" s="5" t="n"/>
       <c r="P286" s="5" t="n"/>
+      <c r="Q286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="5" t="n"/>
@@ -5814,6 +6114,7 @@
       <c r="N287" s="7" t="n"/>
       <c r="O287" s="5" t="n"/>
       <c r="P287" s="5" t="n"/>
+      <c r="Q287" s="5" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="5" t="n"/>
@@ -5832,6 +6133,7 @@
       <c r="N288" s="7" t="n"/>
       <c r="O288" s="5" t="n"/>
       <c r="P288" s="5" t="n"/>
+      <c r="Q288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="5" t="n"/>
@@ -5850,6 +6152,7 @@
       <c r="N289" s="7" t="n"/>
       <c r="O289" s="5" t="n"/>
       <c r="P289" s="5" t="n"/>
+      <c r="Q289" s="5" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="5" t="n"/>
@@ -5868,6 +6171,7 @@
       <c r="N290" s="7" t="n"/>
       <c r="O290" s="5" t="n"/>
       <c r="P290" s="5" t="n"/>
+      <c r="Q290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="5" t="n"/>
@@ -5886,6 +6190,7 @@
       <c r="N291" s="7" t="n"/>
       <c r="O291" s="5" t="n"/>
       <c r="P291" s="5" t="n"/>
+      <c r="Q291" s="5" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="5" t="n"/>
@@ -5904,6 +6209,7 @@
       <c r="N292" s="7" t="n"/>
       <c r="O292" s="5" t="n"/>
       <c r="P292" s="5" t="n"/>
+      <c r="Q292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="5" t="n"/>
@@ -5922,6 +6228,7 @@
       <c r="N293" s="7" t="n"/>
       <c r="O293" s="5" t="n"/>
       <c r="P293" s="5" t="n"/>
+      <c r="Q293" s="5" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="5" t="n"/>
@@ -5940,6 +6247,7 @@
       <c r="N294" s="7" t="n"/>
       <c r="O294" s="5" t="n"/>
       <c r="P294" s="5" t="n"/>
+      <c r="Q294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="5" t="n"/>
@@ -5958,6 +6266,7 @@
       <c r="N295" s="7" t="n"/>
       <c r="O295" s="5" t="n"/>
       <c r="P295" s="5" t="n"/>
+      <c r="Q295" s="5" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="5" t="n"/>
@@ -5976,6 +6285,7 @@
       <c r="N296" s="7" t="n"/>
       <c r="O296" s="5" t="n"/>
       <c r="P296" s="5" t="n"/>
+      <c r="Q296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="5" t="n"/>
@@ -5994,6 +6304,7 @@
       <c r="N297" s="7" t="n"/>
       <c r="O297" s="5" t="n"/>
       <c r="P297" s="5" t="n"/>
+      <c r="Q297" s="5" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="5" t="n"/>
@@ -6012,6 +6323,7 @@
       <c r="N298" s="7" t="n"/>
       <c r="O298" s="5" t="n"/>
       <c r="P298" s="5" t="n"/>
+      <c r="Q298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="5" t="n"/>
@@ -6030,6 +6342,7 @@
       <c r="N299" s="7" t="n"/>
       <c r="O299" s="5" t="n"/>
       <c r="P299" s="5" t="n"/>
+      <c r="Q299" s="5" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="5" t="n"/>
@@ -6048,6 +6361,7 @@
       <c r="N300" s="7" t="n"/>
       <c r="O300" s="5" t="n"/>
       <c r="P300" s="5" t="n"/>
+      <c r="Q300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="5" t="n"/>
@@ -6066,6 +6380,7 @@
       <c r="N301" s="7" t="n"/>
       <c r="O301" s="5" t="n"/>
       <c r="P301" s="5" t="n"/>
+      <c r="Q301" s="5" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="5" t="n"/>
@@ -6084,6 +6399,7 @@
       <c r="N302" s="7" t="n"/>
       <c r="O302" s="5" t="n"/>
       <c r="P302" s="5" t="n"/>
+      <c r="Q302" s="5" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="5" t="n"/>
@@ -6102,6 +6418,7 @@
       <c r="N303" s="7" t="n"/>
       <c r="O303" s="5" t="n"/>
       <c r="P303" s="5" t="n"/>
+      <c r="Q303" s="5" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="5" t="n"/>
@@ -6120,6 +6437,7 @@
       <c r="N304" s="7" t="n"/>
       <c r="O304" s="5" t="n"/>
       <c r="P304" s="5" t="n"/>
+      <c r="Q304" s="5" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="5" t="n"/>
@@ -6138,6 +6456,7 @@
       <c r="N305" s="7" t="n"/>
       <c r="O305" s="5" t="n"/>
       <c r="P305" s="5" t="n"/>
+      <c r="Q305" s="5" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="5" t="n"/>
@@ -6156,6 +6475,7 @@
       <c r="N306" s="7" t="n"/>
       <c r="O306" s="5" t="n"/>
       <c r="P306" s="5" t="n"/>
+      <c r="Q306" s="5" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="5" t="n"/>
@@ -6174,6 +6494,7 @@
       <c r="N307" s="7" t="n"/>
       <c r="O307" s="5" t="n"/>
       <c r="P307" s="5" t="n"/>
+      <c r="Q307" s="5" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="5" t="n"/>
@@ -6192,6 +6513,7 @@
       <c r="N308" s="7" t="n"/>
       <c r="O308" s="5" t="n"/>
       <c r="P308" s="5" t="n"/>
+      <c r="Q308" s="5" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="5" t="n"/>
@@ -6210,6 +6532,7 @@
       <c r="N309" s="7" t="n"/>
       <c r="O309" s="5" t="n"/>
       <c r="P309" s="5" t="n"/>
+      <c r="Q309" s="5" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="5" t="n"/>
@@ -6228,6 +6551,7 @@
       <c r="N310" s="7" t="n"/>
       <c r="O310" s="5" t="n"/>
       <c r="P310" s="5" t="n"/>
+      <c r="Q310" s="5" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="5" t="n"/>
@@ -6246,6 +6570,7 @@
       <c r="N311" s="7" t="n"/>
       <c r="O311" s="5" t="n"/>
       <c r="P311" s="5" t="n"/>
+      <c r="Q311" s="5" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="5" t="n"/>
@@ -6264,6 +6589,7 @@
       <c r="N312" s="7" t="n"/>
       <c r="O312" s="5" t="n"/>
       <c r="P312" s="5" t="n"/>
+      <c r="Q312" s="5" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="5" t="n"/>
@@ -6282,6 +6608,7 @@
       <c r="N313" s="7" t="n"/>
       <c r="O313" s="5" t="n"/>
       <c r="P313" s="5" t="n"/>
+      <c r="Q313" s="5" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="5" t="n"/>
@@ -6300,6 +6627,7 @@
       <c r="N314" s="7" t="n"/>
       <c r="O314" s="5" t="n"/>
       <c r="P314" s="5" t="n"/>
+      <c r="Q314" s="5" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="5" t="n"/>
@@ -6318,6 +6646,7 @@
       <c r="N315" s="7" t="n"/>
       <c r="O315" s="5" t="n"/>
       <c r="P315" s="5" t="n"/>
+      <c r="Q315" s="5" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="5" t="n"/>
@@ -6336,6 +6665,7 @@
       <c r="N316" s="7" t="n"/>
       <c r="O316" s="5" t="n"/>
       <c r="P316" s="5" t="n"/>
+      <c r="Q316" s="5" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="5" t="n"/>
@@ -6354,6 +6684,7 @@
       <c r="N317" s="7" t="n"/>
       <c r="O317" s="5" t="n"/>
       <c r="P317" s="5" t="n"/>
+      <c r="Q317" s="5" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="5" t="n"/>
@@ -6372,6 +6703,7 @@
       <c r="N318" s="7" t="n"/>
       <c r="O318" s="5" t="n"/>
       <c r="P318" s="5" t="n"/>
+      <c r="Q318" s="5" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="5" t="n"/>
@@ -6390,6 +6722,7 @@
       <c r="N319" s="7" t="n"/>
       <c r="O319" s="5" t="n"/>
       <c r="P319" s="5" t="n"/>
+      <c r="Q319" s="5" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="5" t="n"/>
@@ -6408,6 +6741,7 @@
       <c r="N320" s="7" t="n"/>
       <c r="O320" s="5" t="n"/>
       <c r="P320" s="5" t="n"/>
+      <c r="Q320" s="5" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="5" t="n"/>
@@ -6426,6 +6760,7 @@
       <c r="N321" s="7" t="n"/>
       <c r="O321" s="5" t="n"/>
       <c r="P321" s="5" t="n"/>
+      <c r="Q321" s="5" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="5" t="n"/>
@@ -6444,6 +6779,7 @@
       <c r="N322" s="7" t="n"/>
       <c r="O322" s="5" t="n"/>
       <c r="P322" s="5" t="n"/>
+      <c r="Q322" s="5" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="5" t="n"/>
@@ -6462,6 +6798,7 @@
       <c r="N323" s="7" t="n"/>
       <c r="O323" s="5" t="n"/>
       <c r="P323" s="5" t="n"/>
+      <c r="Q323" s="5" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="5" t="n"/>
@@ -6480,6 +6817,7 @@
       <c r="N324" s="7" t="n"/>
       <c r="O324" s="5" t="n"/>
       <c r="P324" s="5" t="n"/>
+      <c r="Q324" s="5" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n"/>
@@ -6498,6 +6836,7 @@
       <c r="N325" s="7" t="n"/>
       <c r="O325" s="5" t="n"/>
       <c r="P325" s="5" t="n"/>
+      <c r="Q325" s="5" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="5" t="n"/>
@@ -6516,6 +6855,7 @@
       <c r="N326" s="7" t="n"/>
       <c r="O326" s="5" t="n"/>
       <c r="P326" s="5" t="n"/>
+      <c r="Q326" s="5" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="5" t="n"/>
@@ -6534,6 +6874,7 @@
       <c r="N327" s="7" t="n"/>
       <c r="O327" s="5" t="n"/>
       <c r="P327" s="5" t="n"/>
+      <c r="Q327" s="5" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="5" t="n"/>
@@ -6552,6 +6893,7 @@
       <c r="N328" s="7" t="n"/>
       <c r="O328" s="5" t="n"/>
       <c r="P328" s="5" t="n"/>
+      <c r="Q328" s="5" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="5" t="n"/>
@@ -6570,6 +6912,7 @@
       <c r="N329" s="7" t="n"/>
       <c r="O329" s="5" t="n"/>
       <c r="P329" s="5" t="n"/>
+      <c r="Q329" s="5" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="5" t="n"/>
@@ -6588,6 +6931,7 @@
       <c r="N330" s="7" t="n"/>
       <c r="O330" s="5" t="n"/>
       <c r="P330" s="5" t="n"/>
+      <c r="Q330" s="5" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="5" t="n"/>
@@ -6606,6 +6950,7 @@
       <c r="N331" s="7" t="n"/>
       <c r="O331" s="5" t="n"/>
       <c r="P331" s="5" t="n"/>
+      <c r="Q331" s="5" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="5" t="n"/>
@@ -6624,6 +6969,7 @@
       <c r="N332" s="7" t="n"/>
       <c r="O332" s="5" t="n"/>
       <c r="P332" s="5" t="n"/>
+      <c r="Q332" s="5" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="5" t="n"/>
@@ -6642,6 +6988,7 @@
       <c r="N333" s="7" t="n"/>
       <c r="O333" s="5" t="n"/>
       <c r="P333" s="5" t="n"/>
+      <c r="Q333" s="5" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="5" t="n"/>
@@ -6660,6 +7007,7 @@
       <c r="N334" s="7" t="n"/>
       <c r="O334" s="5" t="n"/>
       <c r="P334" s="5" t="n"/>
+      <c r="Q334" s="5" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="5" t="n"/>
@@ -6678,6 +7026,7 @@
       <c r="N335" s="7" t="n"/>
       <c r="O335" s="5" t="n"/>
       <c r="P335" s="5" t="n"/>
+      <c r="Q335" s="5" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="5" t="n"/>
@@ -6696,6 +7045,7 @@
       <c r="N336" s="7" t="n"/>
       <c r="O336" s="5" t="n"/>
       <c r="P336" s="5" t="n"/>
+      <c r="Q336" s="5" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="5" t="n"/>
@@ -6714,6 +7064,7 @@
       <c r="N337" s="7" t="n"/>
       <c r="O337" s="5" t="n"/>
       <c r="P337" s="5" t="n"/>
+      <c r="Q337" s="5" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="5" t="n"/>
@@ -6732,6 +7083,7 @@
       <c r="N338" s="7" t="n"/>
       <c r="O338" s="5" t="n"/>
       <c r="P338" s="5" t="n"/>
+      <c r="Q338" s="5" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="5" t="n"/>
@@ -6750,6 +7102,7 @@
       <c r="N339" s="7" t="n"/>
       <c r="O339" s="5" t="n"/>
       <c r="P339" s="5" t="n"/>
+      <c r="Q339" s="5" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="5" t="n"/>
@@ -6768,6 +7121,7 @@
       <c r="N340" s="7" t="n"/>
       <c r="O340" s="5" t="n"/>
       <c r="P340" s="5" t="n"/>
+      <c r="Q340" s="5" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="5" t="n"/>
@@ -6786,6 +7140,7 @@
       <c r="N341" s="7" t="n"/>
       <c r="O341" s="5" t="n"/>
       <c r="P341" s="5" t="n"/>
+      <c r="Q341" s="5" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="5" t="n"/>
@@ -6804,6 +7159,7 @@
       <c r="N342" s="7" t="n"/>
       <c r="O342" s="5" t="n"/>
       <c r="P342" s="5" t="n"/>
+      <c r="Q342" s="5" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="5" t="n"/>
@@ -6822,6 +7178,7 @@
       <c r="N343" s="7" t="n"/>
       <c r="O343" s="5" t="n"/>
       <c r="P343" s="5" t="n"/>
+      <c r="Q343" s="5" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="5" t="n"/>
@@ -6840,6 +7197,7 @@
       <c r="N344" s="7" t="n"/>
       <c r="O344" s="5" t="n"/>
       <c r="P344" s="5" t="n"/>
+      <c r="Q344" s="5" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="5" t="n"/>
@@ -6858,6 +7216,7 @@
       <c r="N345" s="7" t="n"/>
       <c r="O345" s="5" t="n"/>
       <c r="P345" s="5" t="n"/>
+      <c r="Q345" s="5" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="5" t="n"/>
@@ -6876,6 +7235,7 @@
       <c r="N346" s="7" t="n"/>
       <c r="O346" s="5" t="n"/>
       <c r="P346" s="5" t="n"/>
+      <c r="Q346" s="5" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="5" t="n"/>
@@ -6894,6 +7254,7 @@
       <c r="N347" s="7" t="n"/>
       <c r="O347" s="5" t="n"/>
       <c r="P347" s="5" t="n"/>
+      <c r="Q347" s="5" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="5" t="n"/>
@@ -6912,6 +7273,7 @@
       <c r="N348" s="7" t="n"/>
       <c r="O348" s="5" t="n"/>
       <c r="P348" s="5" t="n"/>
+      <c r="Q348" s="5" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="5" t="n"/>
@@ -6930,6 +7292,7 @@
       <c r="N349" s="7" t="n"/>
       <c r="O349" s="5" t="n"/>
       <c r="P349" s="5" t="n"/>
+      <c r="Q349" s="5" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="5" t="n"/>
@@ -6948,6 +7311,7 @@
       <c r="N350" s="7" t="n"/>
       <c r="O350" s="5" t="n"/>
       <c r="P350" s="5" t="n"/>
+      <c r="Q350" s="5" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="5" t="n"/>
@@ -6966,6 +7330,7 @@
       <c r="N351" s="7" t="n"/>
       <c r="O351" s="5" t="n"/>
       <c r="P351" s="5" t="n"/>
+      <c r="Q351" s="5" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="5" t="n"/>
@@ -6984,6 +7349,7 @@
       <c r="N352" s="7" t="n"/>
       <c r="O352" s="5" t="n"/>
       <c r="P352" s="5" t="n"/>
+      <c r="Q352" s="5" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="5" t="n"/>
@@ -7002,6 +7368,7 @@
       <c r="N353" s="7" t="n"/>
       <c r="O353" s="5" t="n"/>
       <c r="P353" s="5" t="n"/>
+      <c r="Q353" s="5" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="5" t="n"/>
@@ -7020,6 +7387,7 @@
       <c r="N354" s="7" t="n"/>
       <c r="O354" s="5" t="n"/>
       <c r="P354" s="5" t="n"/>
+      <c r="Q354" s="5" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="5" t="n"/>
@@ -7038,6 +7406,7 @@
       <c r="N355" s="7" t="n"/>
       <c r="O355" s="5" t="n"/>
       <c r="P355" s="5" t="n"/>
+      <c r="Q355" s="5" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="5" t="n"/>
@@ -7056,6 +7425,7 @@
       <c r="N356" s="7" t="n"/>
       <c r="O356" s="5" t="n"/>
       <c r="P356" s="5" t="n"/>
+      <c r="Q356" s="5" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="5" t="n"/>
@@ -7074,6 +7444,7 @@
       <c r="N357" s="7" t="n"/>
       <c r="O357" s="5" t="n"/>
       <c r="P357" s="5" t="n"/>
+      <c r="Q357" s="5" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="5" t="n"/>
@@ -7092,6 +7463,7 @@
       <c r="N358" s="7" t="n"/>
       <c r="O358" s="5" t="n"/>
       <c r="P358" s="5" t="n"/>
+      <c r="Q358" s="5" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="5" t="n"/>
@@ -7110,6 +7482,7 @@
       <c r="N359" s="7" t="n"/>
       <c r="O359" s="5" t="n"/>
       <c r="P359" s="5" t="n"/>
+      <c r="Q359" s="5" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="5" t="n"/>
@@ -7128,6 +7501,7 @@
       <c r="N360" s="7" t="n"/>
       <c r="O360" s="5" t="n"/>
       <c r="P360" s="5" t="n"/>
+      <c r="Q360" s="5" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="5" t="n"/>
@@ -7146,6 +7520,7 @@
       <c r="N361" s="7" t="n"/>
       <c r="O361" s="5" t="n"/>
       <c r="P361" s="5" t="n"/>
+      <c r="Q361" s="5" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="5" t="n"/>
@@ -7164,6 +7539,7 @@
       <c r="N362" s="7" t="n"/>
       <c r="O362" s="5" t="n"/>
       <c r="P362" s="5" t="n"/>
+      <c r="Q362" s="5" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="5" t="n"/>
@@ -7182,6 +7558,7 @@
       <c r="N363" s="7" t="n"/>
       <c r="O363" s="5" t="n"/>
       <c r="P363" s="5" t="n"/>
+      <c r="Q363" s="5" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="5" t="n"/>
@@ -7200,6 +7577,7 @@
       <c r="N364" s="7" t="n"/>
       <c r="O364" s="5" t="n"/>
       <c r="P364" s="5" t="n"/>
+      <c r="Q364" s="5" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="5" t="n"/>
@@ -7218,6 +7596,7 @@
       <c r="N365" s="7" t="n"/>
       <c r="O365" s="5" t="n"/>
       <c r="P365" s="5" t="n"/>
+      <c r="Q365" s="5" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="5" t="n"/>
@@ -7236,6 +7615,7 @@
       <c r="N366" s="7" t="n"/>
       <c r="O366" s="5" t="n"/>
       <c r="P366" s="5" t="n"/>
+      <c r="Q366" s="5" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="5" t="n"/>
@@ -7254,6 +7634,7 @@
       <c r="N367" s="7" t="n"/>
       <c r="O367" s="5" t="n"/>
       <c r="P367" s="5" t="n"/>
+      <c r="Q367" s="5" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="5" t="n"/>
@@ -7272,6 +7653,7 @@
       <c r="N368" s="7" t="n"/>
       <c r="O368" s="5" t="n"/>
       <c r="P368" s="5" t="n"/>
+      <c r="Q368" s="5" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="5" t="n"/>
@@ -7290,6 +7672,7 @@
       <c r="N369" s="7" t="n"/>
       <c r="O369" s="5" t="n"/>
       <c r="P369" s="5" t="n"/>
+      <c r="Q369" s="5" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="5" t="n"/>
@@ -7308,6 +7691,7 @@
       <c r="N370" s="7" t="n"/>
       <c r="O370" s="5" t="n"/>
       <c r="P370" s="5" t="n"/>
+      <c r="Q370" s="5" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="5" t="n"/>
@@ -7326,6 +7710,7 @@
       <c r="N371" s="7" t="n"/>
       <c r="O371" s="5" t="n"/>
       <c r="P371" s="5" t="n"/>
+      <c r="Q371" s="5" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="5" t="n"/>
@@ -7344,6 +7729,7 @@
       <c r="N372" s="7" t="n"/>
       <c r="O372" s="5" t="n"/>
       <c r="P372" s="5" t="n"/>
+      <c r="Q372" s="5" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="5" t="n"/>
@@ -7362,6 +7748,7 @@
       <c r="N373" s="7" t="n"/>
       <c r="O373" s="5" t="n"/>
       <c r="P373" s="5" t="n"/>
+      <c r="Q373" s="5" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="5" t="n"/>
@@ -7380,6 +7767,7 @@
       <c r="N374" s="7" t="n"/>
       <c r="O374" s="5" t="n"/>
       <c r="P374" s="5" t="n"/>
+      <c r="Q374" s="5" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="5" t="n"/>
@@ -7398,6 +7786,7 @@
       <c r="N375" s="7" t="n"/>
       <c r="O375" s="5" t="n"/>
       <c r="P375" s="5" t="n"/>
+      <c r="Q375" s="5" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="5" t="n"/>
@@ -7416,6 +7805,7 @@
       <c r="N376" s="7" t="n"/>
       <c r="O376" s="5" t="n"/>
       <c r="P376" s="5" t="n"/>
+      <c r="Q376" s="5" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="5" t="n"/>
@@ -7434,6 +7824,7 @@
       <c r="N377" s="7" t="n"/>
       <c r="O377" s="5" t="n"/>
       <c r="P377" s="5" t="n"/>
+      <c r="Q377" s="5" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="5" t="n"/>
@@ -7452,6 +7843,7 @@
       <c r="N378" s="7" t="n"/>
       <c r="O378" s="5" t="n"/>
       <c r="P378" s="5" t="n"/>
+      <c r="Q378" s="5" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="5" t="n"/>
@@ -7470,6 +7862,7 @@
       <c r="N379" s="7" t="n"/>
       <c r="O379" s="5" t="n"/>
       <c r="P379" s="5" t="n"/>
+      <c r="Q379" s="5" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="5" t="n"/>
@@ -7488,6 +7881,7 @@
       <c r="N380" s="7" t="n"/>
       <c r="O380" s="5" t="n"/>
       <c r="P380" s="5" t="n"/>
+      <c r="Q380" s="5" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="5" t="n"/>
@@ -7506,6 +7900,7 @@
       <c r="N381" s="7" t="n"/>
       <c r="O381" s="5" t="n"/>
       <c r="P381" s="5" t="n"/>
+      <c r="Q381" s="5" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="5" t="n"/>
@@ -7524,6 +7919,7 @@
       <c r="N382" s="7" t="n"/>
       <c r="O382" s="5" t="n"/>
       <c r="P382" s="5" t="n"/>
+      <c r="Q382" s="5" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="5" t="n"/>
@@ -7542,6 +7938,7 @@
       <c r="N383" s="7" t="n"/>
       <c r="O383" s="5" t="n"/>
       <c r="P383" s="5" t="n"/>
+      <c r="Q383" s="5" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="5" t="n"/>
@@ -7560,6 +7957,7 @@
       <c r="N384" s="7" t="n"/>
       <c r="O384" s="5" t="n"/>
       <c r="P384" s="5" t="n"/>
+      <c r="Q384" s="5" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="5" t="n"/>
@@ -7578,6 +7976,7 @@
       <c r="N385" s="7" t="n"/>
       <c r="O385" s="5" t="n"/>
       <c r="P385" s="5" t="n"/>
+      <c r="Q385" s="5" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="5" t="n"/>
@@ -7596,6 +7995,7 @@
       <c r="N386" s="7" t="n"/>
       <c r="O386" s="5" t="n"/>
       <c r="P386" s="5" t="n"/>
+      <c r="Q386" s="5" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="5" t="n"/>
@@ -7614,6 +8014,7 @@
       <c r="N387" s="7" t="n"/>
       <c r="O387" s="5" t="n"/>
       <c r="P387" s="5" t="n"/>
+      <c r="Q387" s="5" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="5" t="n"/>
@@ -7632,6 +8033,7 @@
       <c r="N388" s="7" t="n"/>
       <c r="O388" s="5" t="n"/>
       <c r="P388" s="5" t="n"/>
+      <c r="Q388" s="5" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="5" t="n"/>
@@ -7650,6 +8052,7 @@
       <c r="N389" s="7" t="n"/>
       <c r="O389" s="5" t="n"/>
       <c r="P389" s="5" t="n"/>
+      <c r="Q389" s="5" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="5" t="n"/>
@@ -7668,6 +8071,7 @@
       <c r="N390" s="7" t="n"/>
       <c r="O390" s="5" t="n"/>
       <c r="P390" s="5" t="n"/>
+      <c r="Q390" s="5" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="5" t="n"/>
@@ -7686,6 +8090,7 @@
       <c r="N391" s="7" t="n"/>
       <c r="O391" s="5" t="n"/>
       <c r="P391" s="5" t="n"/>
+      <c r="Q391" s="5" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="5" t="n"/>
@@ -7704,6 +8109,7 @@
       <c r="N392" s="7" t="n"/>
       <c r="O392" s="5" t="n"/>
       <c r="P392" s="5" t="n"/>
+      <c r="Q392" s="5" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="5" t="n"/>
@@ -7722,6 +8128,7 @@
       <c r="N393" s="7" t="n"/>
       <c r="O393" s="5" t="n"/>
       <c r="P393" s="5" t="n"/>
+      <c r="Q393" s="5" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="5" t="n"/>
@@ -7740,6 +8147,7 @@
       <c r="N394" s="7" t="n"/>
       <c r="O394" s="5" t="n"/>
       <c r="P394" s="5" t="n"/>
+      <c r="Q394" s="5" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="5" t="n"/>
@@ -7758,6 +8166,7 @@
       <c r="N395" s="7" t="n"/>
       <c r="O395" s="5" t="n"/>
       <c r="P395" s="5" t="n"/>
+      <c r="Q395" s="5" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="5" t="n"/>
@@ -7776,6 +8185,7 @@
       <c r="N396" s="7" t="n"/>
       <c r="O396" s="5" t="n"/>
       <c r="P396" s="5" t="n"/>
+      <c r="Q396" s="5" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="5" t="n"/>
@@ -7794,6 +8204,7 @@
       <c r="N397" s="7" t="n"/>
       <c r="O397" s="5" t="n"/>
       <c r="P397" s="5" t="n"/>
+      <c r="Q397" s="5" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="5" t="n"/>
@@ -7812,6 +8223,7 @@
       <c r="N398" s="7" t="n"/>
       <c r="O398" s="5" t="n"/>
       <c r="P398" s="5" t="n"/>
+      <c r="Q398" s="5" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="5" t="n"/>
@@ -7830,6 +8242,7 @@
       <c r="N399" s="7" t="n"/>
       <c r="O399" s="5" t="n"/>
       <c r="P399" s="5" t="n"/>
+      <c r="Q399" s="5" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="5" t="n"/>
@@ -7848,6 +8261,7 @@
       <c r="N400" s="7" t="n"/>
       <c r="O400" s="5" t="n"/>
       <c r="P400" s="5" t="n"/>
+      <c r="Q400" s="5" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="5" t="n"/>
@@ -7866,6 +8280,7 @@
       <c r="N401" s="7" t="n"/>
       <c r="O401" s="5" t="n"/>
       <c r="P401" s="5" t="n"/>
+      <c r="Q401" s="5" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="5" t="n"/>
@@ -7884,6 +8299,7 @@
       <c r="N402" s="7" t="n"/>
       <c r="O402" s="5" t="n"/>
       <c r="P402" s="5" t="n"/>
+      <c r="Q402" s="5" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="5" t="n"/>
@@ -7902,6 +8318,7 @@
       <c r="N403" s="7" t="n"/>
       <c r="O403" s="5" t="n"/>
       <c r="P403" s="5" t="n"/>
+      <c r="Q403" s="5" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="5" t="n"/>
@@ -7920,6 +8337,7 @@
       <c r="N404" s="7" t="n"/>
       <c r="O404" s="5" t="n"/>
       <c r="P404" s="5" t="n"/>
+      <c r="Q404" s="5" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="5" t="n"/>
@@ -7938,6 +8356,7 @@
       <c r="N405" s="7" t="n"/>
       <c r="O405" s="5" t="n"/>
       <c r="P405" s="5" t="n"/>
+      <c r="Q405" s="5" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="5" t="n"/>
@@ -7956,6 +8375,7 @@
       <c r="N406" s="7" t="n"/>
       <c r="O406" s="5" t="n"/>
       <c r="P406" s="5" t="n"/>
+      <c r="Q406" s="5" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="5" t="n"/>
@@ -7974,6 +8394,7 @@
       <c r="N407" s="7" t="n"/>
       <c r="O407" s="5" t="n"/>
       <c r="P407" s="5" t="n"/>
+      <c r="Q407" s="5" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="5" t="n"/>
@@ -7992,6 +8413,7 @@
       <c r="N408" s="7" t="n"/>
       <c r="O408" s="5" t="n"/>
       <c r="P408" s="5" t="n"/>
+      <c r="Q408" s="5" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="5" t="n"/>
@@ -8010,6 +8432,7 @@
       <c r="N409" s="7" t="n"/>
       <c r="O409" s="5" t="n"/>
       <c r="P409" s="5" t="n"/>
+      <c r="Q409" s="5" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="5" t="n"/>
@@ -8028,6 +8451,7 @@
       <c r="N410" s="7" t="n"/>
       <c r="O410" s="5" t="n"/>
       <c r="P410" s="5" t="n"/>
+      <c r="Q410" s="5" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="5" t="n"/>
@@ -8046,6 +8470,7 @@
       <c r="N411" s="7" t="n"/>
       <c r="O411" s="5" t="n"/>
       <c r="P411" s="5" t="n"/>
+      <c r="Q411" s="5" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="5" t="n"/>
@@ -8064,6 +8489,7 @@
       <c r="N412" s="7" t="n"/>
       <c r="O412" s="5" t="n"/>
       <c r="P412" s="5" t="n"/>
+      <c r="Q412" s="5" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="5" t="n"/>
@@ -8082,6 +8508,7 @@
       <c r="N413" s="7" t="n"/>
       <c r="O413" s="5" t="n"/>
       <c r="P413" s="5" t="n"/>
+      <c r="Q413" s="5" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="5" t="n"/>
@@ -8100,6 +8527,7 @@
       <c r="N414" s="7" t="n"/>
       <c r="O414" s="5" t="n"/>
       <c r="P414" s="5" t="n"/>
+      <c r="Q414" s="5" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="5" t="n"/>
@@ -8118,6 +8546,7 @@
       <c r="N415" s="7" t="n"/>
       <c r="O415" s="5" t="n"/>
       <c r="P415" s="5" t="n"/>
+      <c r="Q415" s="5" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="5" t="n"/>
@@ -8136,6 +8565,7 @@
       <c r="N416" s="7" t="n"/>
       <c r="O416" s="5" t="n"/>
       <c r="P416" s="5" t="n"/>
+      <c r="Q416" s="5" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="5" t="n"/>
@@ -8154,6 +8584,7 @@
       <c r="N417" s="7" t="n"/>
       <c r="O417" s="5" t="n"/>
       <c r="P417" s="5" t="n"/>
+      <c r="Q417" s="5" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="5" t="n"/>
@@ -8172,6 +8603,7 @@
       <c r="N418" s="7" t="n"/>
       <c r="O418" s="5" t="n"/>
       <c r="P418" s="5" t="n"/>
+      <c r="Q418" s="5" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="5" t="n"/>
@@ -8190,6 +8622,7 @@
       <c r="N419" s="7" t="n"/>
       <c r="O419" s="5" t="n"/>
       <c r="P419" s="5" t="n"/>
+      <c r="Q419" s="5" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="5" t="n"/>
@@ -8208,6 +8641,7 @@
       <c r="N420" s="7" t="n"/>
       <c r="O420" s="5" t="n"/>
       <c r="P420" s="5" t="n"/>
+      <c r="Q420" s="5" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="5" t="n"/>
@@ -8226,6 +8660,7 @@
       <c r="N421" s="7" t="n"/>
       <c r="O421" s="5" t="n"/>
       <c r="P421" s="5" t="n"/>
+      <c r="Q421" s="5" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="5" t="n"/>
@@ -8244,6 +8679,7 @@
       <c r="N422" s="7" t="n"/>
       <c r="O422" s="5" t="n"/>
       <c r="P422" s="5" t="n"/>
+      <c r="Q422" s="5" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="5" t="n"/>
@@ -8262,6 +8698,7 @@
       <c r="N423" s="7" t="n"/>
       <c r="O423" s="5" t="n"/>
       <c r="P423" s="5" t="n"/>
+      <c r="Q423" s="5" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="5" t="n"/>
@@ -8280,6 +8717,7 @@
       <c r="N424" s="7" t="n"/>
       <c r="O424" s="5" t="n"/>
       <c r="P424" s="5" t="n"/>
+      <c r="Q424" s="5" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="5" t="n"/>
@@ -8298,6 +8736,7 @@
       <c r="N425" s="7" t="n"/>
       <c r="O425" s="5" t="n"/>
       <c r="P425" s="5" t="n"/>
+      <c r="Q425" s="5" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="5" t="n"/>
@@ -8316,6 +8755,7 @@
       <c r="N426" s="7" t="n"/>
       <c r="O426" s="5" t="n"/>
       <c r="P426" s="5" t="n"/>
+      <c r="Q426" s="5" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="5" t="n"/>
@@ -8334,6 +8774,7 @@
       <c r="N427" s="7" t="n"/>
       <c r="O427" s="5" t="n"/>
       <c r="P427" s="5" t="n"/>
+      <c r="Q427" s="5" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="5" t="n"/>
@@ -8352,6 +8793,7 @@
       <c r="N428" s="7" t="n"/>
       <c r="O428" s="5" t="n"/>
       <c r="P428" s="5" t="n"/>
+      <c r="Q428" s="5" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="5" t="n"/>
@@ -8370,6 +8812,7 @@
       <c r="N429" s="7" t="n"/>
       <c r="O429" s="5" t="n"/>
       <c r="P429" s="5" t="n"/>
+      <c r="Q429" s="5" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="5" t="n"/>
@@ -8388,6 +8831,7 @@
       <c r="N430" s="7" t="n"/>
       <c r="O430" s="5" t="n"/>
       <c r="P430" s="5" t="n"/>
+      <c r="Q430" s="5" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="5" t="n"/>
@@ -8406,6 +8850,7 @@
       <c r="N431" s="7" t="n"/>
       <c r="O431" s="5" t="n"/>
       <c r="P431" s="5" t="n"/>
+      <c r="Q431" s="5" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="5" t="n"/>
@@ -8424,6 +8869,7 @@
       <c r="N432" s="7" t="n"/>
       <c r="O432" s="5" t="n"/>
       <c r="P432" s="5" t="n"/>
+      <c r="Q432" s="5" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="5" t="n"/>
@@ -8442,6 +8888,7 @@
       <c r="N433" s="7" t="n"/>
       <c r="O433" s="5" t="n"/>
       <c r="P433" s="5" t="n"/>
+      <c r="Q433" s="5" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="5" t="n"/>
@@ -8460,6 +8907,7 @@
       <c r="N434" s="7" t="n"/>
       <c r="O434" s="5" t="n"/>
       <c r="P434" s="5" t="n"/>
+      <c r="Q434" s="5" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="5" t="n"/>
@@ -8478,6 +8926,7 @@
       <c r="N435" s="7" t="n"/>
       <c r="O435" s="5" t="n"/>
       <c r="P435" s="5" t="n"/>
+      <c r="Q435" s="5" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="5" t="n"/>
@@ -8496,6 +8945,7 @@
       <c r="N436" s="7" t="n"/>
       <c r="O436" s="5" t="n"/>
       <c r="P436" s="5" t="n"/>
+      <c r="Q436" s="5" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="5" t="n"/>
@@ -8514,6 +8964,7 @@
       <c r="N437" s="7" t="n"/>
       <c r="O437" s="5" t="n"/>
       <c r="P437" s="5" t="n"/>
+      <c r="Q437" s="5" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="5" t="n"/>
@@ -8532,6 +8983,7 @@
       <c r="N438" s="7" t="n"/>
       <c r="O438" s="5" t="n"/>
       <c r="P438" s="5" t="n"/>
+      <c r="Q438" s="5" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="5" t="n"/>
@@ -8550,6 +9002,7 @@
       <c r="N439" s="7" t="n"/>
       <c r="O439" s="5" t="n"/>
       <c r="P439" s="5" t="n"/>
+      <c r="Q439" s="5" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="5" t="n"/>
@@ -8568,6 +9021,7 @@
       <c r="N440" s="7" t="n"/>
       <c r="O440" s="5" t="n"/>
       <c r="P440" s="5" t="n"/>
+      <c r="Q440" s="5" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="5" t="n"/>
@@ -8586,6 +9040,7 @@
       <c r="N441" s="7" t="n"/>
       <c r="O441" s="5" t="n"/>
       <c r="P441" s="5" t="n"/>
+      <c r="Q441" s="5" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="5" t="n"/>
@@ -8604,6 +9059,7 @@
       <c r="N442" s="7" t="n"/>
       <c r="O442" s="5" t="n"/>
       <c r="P442" s="5" t="n"/>
+      <c r="Q442" s="5" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="5" t="n"/>
@@ -8622,6 +9078,7 @@
       <c r="N443" s="7" t="n"/>
       <c r="O443" s="5" t="n"/>
       <c r="P443" s="5" t="n"/>
+      <c r="Q443" s="5" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="5" t="n"/>
@@ -8640,6 +9097,7 @@
       <c r="N444" s="7" t="n"/>
       <c r="O444" s="5" t="n"/>
       <c r="P444" s="5" t="n"/>
+      <c r="Q444" s="5" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="5" t="n"/>
@@ -8658,6 +9116,7 @@
       <c r="N445" s="7" t="n"/>
       <c r="O445" s="5" t="n"/>
       <c r="P445" s="5" t="n"/>
+      <c r="Q445" s="5" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="5" t="n"/>
@@ -8676,6 +9135,7 @@
       <c r="N446" s="7" t="n"/>
       <c r="O446" s="5" t="n"/>
       <c r="P446" s="5" t="n"/>
+      <c r="Q446" s="5" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="5" t="n"/>
@@ -8694,6 +9154,7 @@
       <c r="N447" s="7" t="n"/>
       <c r="O447" s="5" t="n"/>
       <c r="P447" s="5" t="n"/>
+      <c r="Q447" s="5" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="5" t="n"/>
@@ -8712,6 +9173,7 @@
       <c r="N448" s="7" t="n"/>
       <c r="O448" s="5" t="n"/>
       <c r="P448" s="5" t="n"/>
+      <c r="Q448" s="5" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="5" t="n"/>
@@ -8730,6 +9192,7 @@
       <c r="N449" s="7" t="n"/>
       <c r="O449" s="5" t="n"/>
       <c r="P449" s="5" t="n"/>
+      <c r="Q449" s="5" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="5" t="n"/>
@@ -8748,6 +9211,7 @@
       <c r="N450" s="7" t="n"/>
       <c r="O450" s="5" t="n"/>
       <c r="P450" s="5" t="n"/>
+      <c r="Q450" s="5" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="5" t="n"/>
@@ -8766,6 +9230,7 @@
       <c r="N451" s="7" t="n"/>
       <c r="O451" s="5" t="n"/>
       <c r="P451" s="5" t="n"/>
+      <c r="Q451" s="5" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="5" t="n"/>
@@ -8784,6 +9249,7 @@
       <c r="N452" s="7" t="n"/>
       <c r="O452" s="5" t="n"/>
       <c r="P452" s="5" t="n"/>
+      <c r="Q452" s="5" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="5" t="n"/>
@@ -8802,6 +9268,7 @@
       <c r="N453" s="7" t="n"/>
       <c r="O453" s="5" t="n"/>
       <c r="P453" s="5" t="n"/>
+      <c r="Q453" s="5" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="5" t="n"/>
@@ -8820,6 +9287,7 @@
       <c r="N454" s="7" t="n"/>
       <c r="O454" s="5" t="n"/>
       <c r="P454" s="5" t="n"/>
+      <c r="Q454" s="5" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="5" t="n"/>
@@ -8838,6 +9306,7 @@
       <c r="N455" s="7" t="n"/>
       <c r="O455" s="5" t="n"/>
       <c r="P455" s="5" t="n"/>
+      <c r="Q455" s="5" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="5" t="n"/>
@@ -8856,6 +9325,7 @@
       <c r="N456" s="7" t="n"/>
       <c r="O456" s="5" t="n"/>
       <c r="P456" s="5" t="n"/>
+      <c r="Q456" s="5" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="5" t="n"/>
@@ -8874,6 +9344,7 @@
       <c r="N457" s="7" t="n"/>
       <c r="O457" s="5" t="n"/>
       <c r="P457" s="5" t="n"/>
+      <c r="Q457" s="5" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="5" t="n"/>
@@ -8892,6 +9363,7 @@
       <c r="N458" s="7" t="n"/>
       <c r="O458" s="5" t="n"/>
       <c r="P458" s="5" t="n"/>
+      <c r="Q458" s="5" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="5" t="n"/>
@@ -8910,6 +9382,7 @@
       <c r="N459" s="7" t="n"/>
       <c r="O459" s="5" t="n"/>
       <c r="P459" s="5" t="n"/>
+      <c r="Q459" s="5" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="5" t="n"/>
@@ -8928,6 +9401,7 @@
       <c r="N460" s="7" t="n"/>
       <c r="O460" s="5" t="n"/>
       <c r="P460" s="5" t="n"/>
+      <c r="Q460" s="5" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="5" t="n"/>
@@ -8946,6 +9420,7 @@
       <c r="N461" s="7" t="n"/>
       <c r="O461" s="5" t="n"/>
       <c r="P461" s="5" t="n"/>
+      <c r="Q461" s="5" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="5" t="n"/>
@@ -8964,6 +9439,7 @@
       <c r="N462" s="7" t="n"/>
       <c r="O462" s="5" t="n"/>
       <c r="P462" s="5" t="n"/>
+      <c r="Q462" s="5" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="5" t="n"/>
@@ -8982,6 +9458,7 @@
       <c r="N463" s="7" t="n"/>
       <c r="O463" s="5" t="n"/>
       <c r="P463" s="5" t="n"/>
+      <c r="Q463" s="5" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="5" t="n"/>
@@ -9000,6 +9477,7 @@
       <c r="N464" s="7" t="n"/>
       <c r="O464" s="5" t="n"/>
       <c r="P464" s="5" t="n"/>
+      <c r="Q464" s="5" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="5" t="n"/>
@@ -9018,6 +9496,7 @@
       <c r="N465" s="7" t="n"/>
       <c r="O465" s="5" t="n"/>
       <c r="P465" s="5" t="n"/>
+      <c r="Q465" s="5" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="5" t="n"/>
@@ -9036,6 +9515,7 @@
       <c r="N466" s="7" t="n"/>
       <c r="O466" s="5" t="n"/>
       <c r="P466" s="5" t="n"/>
+      <c r="Q466" s="5" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="5" t="n"/>
@@ -9054,6 +9534,7 @@
       <c r="N467" s="7" t="n"/>
       <c r="O467" s="5" t="n"/>
       <c r="P467" s="5" t="n"/>
+      <c r="Q467" s="5" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="5" t="n"/>
@@ -9072,6 +9553,7 @@
       <c r="N468" s="7" t="n"/>
       <c r="O468" s="5" t="n"/>
       <c r="P468" s="5" t="n"/>
+      <c r="Q468" s="5" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="5" t="n"/>
@@ -9090,6 +9572,7 @@
       <c r="N469" s="7" t="n"/>
       <c r="O469" s="5" t="n"/>
       <c r="P469" s="5" t="n"/>
+      <c r="Q469" s="5" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="5" t="n"/>
@@ -9108,6 +9591,7 @@
       <c r="N470" s="7" t="n"/>
       <c r="O470" s="5" t="n"/>
       <c r="P470" s="5" t="n"/>
+      <c r="Q470" s="5" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="5" t="n"/>
@@ -9126,6 +9610,7 @@
       <c r="N471" s="7" t="n"/>
       <c r="O471" s="5" t="n"/>
       <c r="P471" s="5" t="n"/>
+      <c r="Q471" s="5" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="5" t="n"/>
@@ -9144,6 +9629,7 @@
       <c r="N472" s="7" t="n"/>
       <c r="O472" s="5" t="n"/>
       <c r="P472" s="5" t="n"/>
+      <c r="Q472" s="5" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="5" t="n"/>
@@ -9162,6 +9648,7 @@
       <c r="N473" s="7" t="n"/>
       <c r="O473" s="5" t="n"/>
       <c r="P473" s="5" t="n"/>
+      <c r="Q473" s="5" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="5" t="n"/>
@@ -9180,6 +9667,7 @@
       <c r="N474" s="7" t="n"/>
       <c r="O474" s="5" t="n"/>
       <c r="P474" s="5" t="n"/>
+      <c r="Q474" s="5" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="5" t="n"/>
@@ -9198,6 +9686,7 @@
       <c r="N475" s="7" t="n"/>
       <c r="O475" s="5" t="n"/>
       <c r="P475" s="5" t="n"/>
+      <c r="Q475" s="5" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="5" t="n"/>
@@ -9216,6 +9705,7 @@
       <c r="N476" s="7" t="n"/>
       <c r="O476" s="5" t="n"/>
       <c r="P476" s="5" t="n"/>
+      <c r="Q476" s="5" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="5" t="n"/>
@@ -9234,6 +9724,7 @@
       <c r="N477" s="7" t="n"/>
       <c r="O477" s="5" t="n"/>
       <c r="P477" s="5" t="n"/>
+      <c r="Q477" s="5" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="5" t="n"/>
@@ -9252,6 +9743,7 @@
       <c r="N478" s="7" t="n"/>
       <c r="O478" s="5" t="n"/>
       <c r="P478" s="5" t="n"/>
+      <c r="Q478" s="5" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="5" t="n"/>
@@ -9270,6 +9762,7 @@
       <c r="N479" s="7" t="n"/>
       <c r="O479" s="5" t="n"/>
       <c r="P479" s="5" t="n"/>
+      <c r="Q479" s="5" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="5" t="n"/>
@@ -9288,6 +9781,7 @@
       <c r="N480" s="7" t="n"/>
       <c r="O480" s="5" t="n"/>
       <c r="P480" s="5" t="n"/>
+      <c r="Q480" s="5" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="5" t="n"/>
@@ -9306,6 +9800,7 @@
       <c r="N481" s="7" t="n"/>
       <c r="O481" s="5" t="n"/>
       <c r="P481" s="5" t="n"/>
+      <c r="Q481" s="5" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="5" t="n"/>
@@ -9324,6 +9819,7 @@
       <c r="N482" s="7" t="n"/>
       <c r="O482" s="5" t="n"/>
       <c r="P482" s="5" t="n"/>
+      <c r="Q482" s="5" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="5" t="n"/>
@@ -9342,6 +9838,7 @@
       <c r="N483" s="7" t="n"/>
       <c r="O483" s="5" t="n"/>
       <c r="P483" s="5" t="n"/>
+      <c r="Q483" s="5" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="5" t="n"/>
@@ -9360,6 +9857,7 @@
       <c r="N484" s="7" t="n"/>
       <c r="O484" s="5" t="n"/>
       <c r="P484" s="5" t="n"/>
+      <c r="Q484" s="5" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="5" t="n"/>
@@ -9378,6 +9876,7 @@
       <c r="N485" s="7" t="n"/>
       <c r="O485" s="5" t="n"/>
       <c r="P485" s="5" t="n"/>
+      <c r="Q485" s="5" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="5" t="n"/>
@@ -9396,6 +9895,7 @@
       <c r="N486" s="7" t="n"/>
       <c r="O486" s="5" t="n"/>
       <c r="P486" s="5" t="n"/>
+      <c r="Q486" s="5" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="5" t="n"/>
@@ -9414,6 +9914,7 @@
       <c r="N487" s="7" t="n"/>
       <c r="O487" s="5" t="n"/>
       <c r="P487" s="5" t="n"/>
+      <c r="Q487" s="5" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="5" t="n"/>
@@ -9432,6 +9933,7 @@
       <c r="N488" s="7" t="n"/>
       <c r="O488" s="5" t="n"/>
       <c r="P488" s="5" t="n"/>
+      <c r="Q488" s="5" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="5" t="n"/>
@@ -9450,6 +9952,7 @@
       <c r="N489" s="7" t="n"/>
       <c r="O489" s="5" t="n"/>
       <c r="P489" s="5" t="n"/>
+      <c r="Q489" s="5" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="5" t="n"/>
@@ -9468,6 +9971,7 @@
       <c r="N490" s="7" t="n"/>
       <c r="O490" s="5" t="n"/>
       <c r="P490" s="5" t="n"/>
+      <c r="Q490" s="5" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="5" t="n"/>
@@ -9486,6 +9990,7 @@
       <c r="N491" s="7" t="n"/>
       <c r="O491" s="5" t="n"/>
       <c r="P491" s="5" t="n"/>
+      <c r="Q491" s="5" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="5" t="n"/>
@@ -9504,6 +10009,7 @@
       <c r="N492" s="7" t="n"/>
       <c r="O492" s="5" t="n"/>
       <c r="P492" s="5" t="n"/>
+      <c r="Q492" s="5" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="5" t="n"/>
@@ -9522,6 +10028,7 @@
       <c r="N493" s="7" t="n"/>
       <c r="O493" s="5" t="n"/>
       <c r="P493" s="5" t="n"/>
+      <c r="Q493" s="5" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="5" t="n"/>
@@ -9540,6 +10047,7 @@
       <c r="N494" s="7" t="n"/>
       <c r="O494" s="5" t="n"/>
       <c r="P494" s="5" t="n"/>
+      <c r="Q494" s="5" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="5" t="n"/>
@@ -9558,6 +10066,7 @@
       <c r="N495" s="7" t="n"/>
       <c r="O495" s="5" t="n"/>
       <c r="P495" s="5" t="n"/>
+      <c r="Q495" s="5" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="5" t="n"/>
@@ -9576,6 +10085,7 @@
       <c r="N496" s="7" t="n"/>
       <c r="O496" s="5" t="n"/>
       <c r="P496" s="5" t="n"/>
+      <c r="Q496" s="5" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="5" t="n"/>
@@ -9594,6 +10104,7 @@
       <c r="N497" s="7" t="n"/>
       <c r="O497" s="5" t="n"/>
       <c r="P497" s="5" t="n"/>
+      <c r="Q497" s="5" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="5" t="n"/>
@@ -9612,6 +10123,7 @@
       <c r="N498" s="7" t="n"/>
       <c r="O498" s="5" t="n"/>
       <c r="P498" s="5" t="n"/>
+      <c r="Q498" s="5" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="5" t="n"/>
@@ -9630,6 +10142,7 @@
       <c r="N499" s="7" t="n"/>
       <c r="O499" s="5" t="n"/>
       <c r="P499" s="5" t="n"/>
+      <c r="Q499" s="5" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="5" t="n"/>
@@ -9648,6 +10161,7 @@
       <c r="N500" s="7" t="n"/>
       <c r="O500" s="5" t="n"/>
       <c r="P500" s="5" t="n"/>
+      <c r="Q500" s="5" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="5" t="n"/>
@@ -9666,16 +10180,20 @@
       <c r="N501" s="7" t="n"/>
       <c r="O501" s="5" t="n"/>
       <c r="P501" s="5" t="n"/>
+      <c r="Q501" s="5" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"M.,Mme,M. et Mme"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Courrier,Email,Les deux"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>